<commit_message>
Planning looks working with no blocking inserts
</commit_message>
<xml_diff>
--- a/data/personnes.xlsx
+++ b/data/personnes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sschies1\_code\1.09_VScode\06_VoeuxConcerts\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CE5574F-B8AF-416B-94A0-920C489BCA21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E7411FD-7909-44B5-B000-5B817AA182E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="4">
   <si>
     <t>Nom</t>
   </si>
@@ -67,150 +67,6 @@
   </si>
   <si>
     <t>Tous</t>
-  </si>
-  <si>
-    <t>Bar, Vestiaire, Technique</t>
-  </si>
-  <si>
-    <t>Sécurité, Vestiaire, Billetterie, Accueil</t>
-  </si>
-  <si>
-    <t>Accueil, Technique, Vestiaire</t>
-  </si>
-  <si>
-    <t>Technique, Billetterie</t>
-  </si>
-  <si>
-    <t>Sécurité, Technique, Bar, Billetterie</t>
-  </si>
-  <si>
-    <t>Bar, Billetterie, Technique, Sécurité</t>
-  </si>
-  <si>
-    <t>Sécurité, Accueil, Technique, Bar</t>
-  </si>
-  <si>
-    <t>Billetterie, Bar, Accueil</t>
-  </si>
-  <si>
-    <t>Bar, Billetterie, Vestiaire</t>
-  </si>
-  <si>
-    <t>Bar, Sécurité, Accueil, Technique</t>
-  </si>
-  <si>
-    <t>Technique, Accueil, Billetterie</t>
-  </si>
-  <si>
-    <t>Technique, Sécurité</t>
-  </si>
-  <si>
-    <t>Sécurité, Billetterie, Bar</t>
-  </si>
-  <si>
-    <t>Bar, Sécurité, Vestiaire, Billetterie</t>
-  </si>
-  <si>
-    <t>Accueil, Vestiaire</t>
-  </si>
-  <si>
-    <t>Accueil, Bar</t>
-  </si>
-  <si>
-    <t>Bar, Billetterie, Vestiaire, Technique</t>
-  </si>
-  <si>
-    <t>Accueil, Technique, Sécurité, Bar</t>
-  </si>
-  <si>
-    <t>Accueil, Bar, Billetterie, Vestiaire</t>
-  </si>
-  <si>
-    <t>Bar, Accueil, Technique</t>
-  </si>
-  <si>
-    <t>Technique, Accueil</t>
-  </si>
-  <si>
-    <t>Vestiaire, Sécurité, Billetterie, Accueil</t>
-  </si>
-  <si>
-    <t>Vestiaire, Accueil</t>
-  </si>
-  <si>
-    <t>Vestiaire, Billetterie, Bar</t>
-  </si>
-  <si>
-    <t>Accueil, Vestiaire, Technique, Billetterie</t>
-  </si>
-  <si>
-    <t>Bar, Technique, Billetterie</t>
-  </si>
-  <si>
-    <t>Billetterie, Vestiaire, Bar, Technique</t>
-  </si>
-  <si>
-    <t>Bar, Sécurité, Vestiaire</t>
-  </si>
-  <si>
-    <t>Bar, Accueil, Sécurité, Billetterie</t>
-  </si>
-  <si>
-    <t>Vestiaire, Sécurité, Accueil</t>
-  </si>
-  <si>
-    <t>Billetterie, Bar, Accueil, Sécurité</t>
-  </si>
-  <si>
-    <t>Bar, Sécurité, Technique, Vestiaire</t>
-  </si>
-  <si>
-    <t>Technique, Bar, Billetterie</t>
-  </si>
-  <si>
-    <t>Vestiaire, Billetterie, Bar, Sécurité</t>
-  </si>
-  <si>
-    <t>Bar, Technique</t>
-  </si>
-  <si>
-    <t>Sécurité, Bar, Vestiaire, Billetterie</t>
-  </si>
-  <si>
-    <t>Sécurité, Vestiaire</t>
-  </si>
-  <si>
-    <t>Billetterie, Accueil, Bar, Vestiaire</t>
-  </si>
-  <si>
-    <t>Bar, Accueil, Billetterie, Technique</t>
-  </si>
-  <si>
-    <t>Sécurité, Accueil, Vestiaire</t>
-  </si>
-  <si>
-    <t>Sécurité, Billetterie, Vestiaire, Technique</t>
-  </si>
-  <si>
-    <t>Vestiaire, Billetterie</t>
-  </si>
-  <si>
-    <t>Sécurité, Vestiaire, Accueil, Bar</t>
-  </si>
-  <si>
-    <t>Sécurité, Vestiaire, Technique, Accueil</t>
-  </si>
-  <si>
-    <t>Vestiaire, Bar, Billetterie</t>
-  </si>
-  <si>
-    <t>Sécurité, Vestiaire, Billetterie</t>
-  </si>
-  <si>
-    <t>Technique, Bar</t>
-  </si>
-  <si>
-    <t>Bar, Sécurité, Accueil</t>
   </si>
   <si>
     <t>Prénom</t>
@@ -1645,7 +1501,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>51</v>
+        <v>3</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -1671,7 +1527,7 @@
         <v>Alegria Lily</v>
       </c>
       <c r="C3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.4">
@@ -1682,7 +1538,7 @@
         <v>Alexandra</v>
       </c>
       <c r="C4" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.4">
@@ -1704,7 +1560,7 @@
         <v>Analou</v>
       </c>
       <c r="C6" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.4">
@@ -1726,7 +1582,7 @@
         <v>Annouk</v>
       </c>
       <c r="C8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.4">
@@ -1748,7 +1604,7 @@
         <v>Arsène</v>
       </c>
       <c r="C10" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.4">
@@ -1759,7 +1615,7 @@
         <v>Arthur</v>
       </c>
       <c r="C11" t="s">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.4">
@@ -1781,7 +1637,7 @@
         <v>Auxence</v>
       </c>
       <c r="C13" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.4">
@@ -1792,7 +1648,7 @@
         <v>Ava</v>
       </c>
       <c r="C14" t="s">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.4">
@@ -1803,7 +1659,7 @@
         <v>Benoît</v>
       </c>
       <c r="C15" t="s">
-        <v>11</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.4">
@@ -1814,7 +1670,7 @@
         <v>Corentin</v>
       </c>
       <c r="C16" t="s">
-        <v>12</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.4">
@@ -1825,7 +1681,7 @@
         <v>Emma</v>
       </c>
       <c r="C17" t="s">
-        <v>13</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.4">
@@ -1836,7 +1692,7 @@
         <v>Enzo</v>
       </c>
       <c r="C18" t="s">
-        <v>14</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.4">
@@ -1847,7 +1703,7 @@
         <v>Eugénie</v>
       </c>
       <c r="C19" t="s">
-        <v>15</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.4">
@@ -1858,7 +1714,7 @@
         <v>Iris</v>
       </c>
       <c r="C20" t="s">
-        <v>16</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.4">
@@ -1869,7 +1725,7 @@
         <v>Jamilah</v>
       </c>
       <c r="C21" t="s">
-        <v>17</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.4">
@@ -1880,7 +1736,7 @@
         <v>Jolan</v>
       </c>
       <c r="C22" t="s">
-        <v>18</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.4">
@@ -1891,7 +1747,7 @@
         <v xml:space="preserve">Jonas </v>
       </c>
       <c r="C23" t="s">
-        <v>19</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.4">
@@ -1902,7 +1758,7 @@
         <v>Jules</v>
       </c>
       <c r="C24" t="s">
-        <v>20</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.4">
@@ -1913,7 +1769,7 @@
         <v>Julie</v>
       </c>
       <c r="C25" t="s">
-        <v>21</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.4">
@@ -1924,7 +1780,7 @@
         <v>Kristel</v>
       </c>
       <c r="C26" t="s">
-        <v>22</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.4">
@@ -1935,7 +1791,7 @@
         <v>Léa</v>
       </c>
       <c r="C27" t="s">
-        <v>23</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.4">
@@ -1946,7 +1802,7 @@
         <v>Léa</v>
       </c>
       <c r="C28" t="s">
-        <v>24</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.4">
@@ -1957,7 +1813,7 @@
         <v>Lina-Rosa</v>
       </c>
       <c r="C29" t="s">
-        <v>25</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.4">
@@ -1968,7 +1824,7 @@
         <v>Lisa</v>
       </c>
       <c r="C30" t="s">
-        <v>26</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.4">
@@ -1979,7 +1835,7 @@
         <v>Lisa</v>
       </c>
       <c r="C31" t="s">
-        <v>27</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.4">
@@ -1990,7 +1846,7 @@
         <v>Louis</v>
       </c>
       <c r="C32" t="s">
-        <v>28</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.4">
@@ -2001,7 +1857,7 @@
         <v>Louis</v>
       </c>
       <c r="C33" t="s">
-        <v>29</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.4">
@@ -2012,7 +1868,7 @@
         <v>Louise</v>
       </c>
       <c r="C34" t="s">
-        <v>30</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.4">
@@ -2023,7 +1879,7 @@
         <v>Lucas</v>
       </c>
       <c r="C35" t="s">
-        <v>31</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.4">
@@ -2034,7 +1890,7 @@
         <v>Lucie</v>
       </c>
       <c r="C36" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.4">
@@ -2045,7 +1901,7 @@
         <v>Maëlan</v>
       </c>
       <c r="C37" t="s">
-        <v>32</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.4">
@@ -2056,7 +1912,7 @@
         <v>Maëlle</v>
       </c>
       <c r="C38" t="s">
-        <v>33</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.4">
@@ -2078,7 +1934,7 @@
         <v>Marot</v>
       </c>
       <c r="C40" t="s">
-        <v>34</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.4">
@@ -2089,7 +1945,7 @@
         <v>Mathis</v>
       </c>
       <c r="C41" t="s">
-        <v>34</v>
+        <v>2</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.4">
@@ -2100,7 +1956,7 @@
         <v>Matteo</v>
       </c>
       <c r="C42" t="s">
-        <v>35</v>
+        <v>2</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.4">
@@ -2111,7 +1967,7 @@
         <v>Maxime</v>
       </c>
       <c r="C43" t="s">
-        <v>36</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.4">
@@ -2122,7 +1978,7 @@
         <v>Maya</v>
       </c>
       <c r="C44" t="s">
-        <v>37</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.4">
@@ -2133,7 +1989,7 @@
         <v>Mickaël</v>
       </c>
       <c r="C45" t="s">
-        <v>38</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.4">
@@ -2144,7 +2000,7 @@
         <v>Morgana</v>
       </c>
       <c r="C46" t="s">
-        <v>39</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.4">
@@ -2155,7 +2011,7 @@
         <v>Morgane</v>
       </c>
       <c r="C47" t="s">
-        <v>40</v>
+        <v>2</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.4">
@@ -2166,7 +2022,7 @@
         <v>Nathalia</v>
       </c>
       <c r="C48" t="s">
-        <v>41</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.4">
@@ -2188,7 +2044,7 @@
         <v>Patrick</v>
       </c>
       <c r="C50" t="s">
-        <v>42</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.4">
@@ -2199,7 +2055,7 @@
         <v>Rama</v>
       </c>
       <c r="C51" t="s">
-        <v>43</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.4">
@@ -2210,7 +2066,7 @@
         <v>Raphaël</v>
       </c>
       <c r="C52" t="s">
-        <v>23</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.4">
@@ -2221,7 +2077,7 @@
         <v>Raphaëlle</v>
       </c>
       <c r="C53" t="s">
-        <v>44</v>
+        <v>2</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.4">
@@ -2232,7 +2088,7 @@
         <v>Roxanne</v>
       </c>
       <c r="C54" t="s">
-        <v>45</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.4">
@@ -2243,7 +2099,7 @@
         <v>Sébastien</v>
       </c>
       <c r="C55" t="s">
-        <v>44</v>
+        <v>2</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.4">
@@ -2254,7 +2110,7 @@
         <v>Simon</v>
       </c>
       <c r="C56" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.4">
@@ -2265,7 +2121,7 @@
         <v>Theo</v>
       </c>
       <c r="C57" t="s">
-        <v>46</v>
+        <v>2</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.4">
@@ -2276,7 +2132,7 @@
         <v>Thibault</v>
       </c>
       <c r="C58" t="s">
-        <v>47</v>
+        <v>2</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.4">
@@ -2287,7 +2143,7 @@
         <v>Titouan</v>
       </c>
       <c r="C59" t="s">
-        <v>48</v>
+        <v>2</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.4">
@@ -2298,7 +2154,7 @@
         <v>Tristan</v>
       </c>
       <c r="C60" t="s">
-        <v>49</v>
+        <v>2</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.4">
@@ -2309,7 +2165,7 @@
         <v>Yann</v>
       </c>
       <c r="C61" t="s">
-        <v>50</v>
+        <v>2</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.4">
@@ -2320,7 +2176,7 @@
         <v>Ysatis</v>
       </c>
       <c r="C62" t="s">
-        <v>44</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Dry run with blocages.xlsx
</commit_message>
<xml_diff>
--- a/data/personnes.xlsx
+++ b/data/personnes.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sschies1\_code\1.09_VScode\06_VoeuxConcerts\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FAE588F-3FB6-4F43-829E-F6BDA5079D92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9FE3BF7-536A-4DFD-BACE-E02E255DAA87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="15">
   <si>
     <t>Nom</t>
   </si>
@@ -78,9 +78,6 @@
     <t>Accueil</t>
   </si>
   <si>
-    <t>Bourdon.e</t>
-  </si>
-  <si>
     <t>Horaires</t>
   </si>
   <si>
@@ -88,6 +85,24 @@
   </si>
   <si>
     <t>Bar public</t>
+  </si>
+  <si>
+    <t>Bourdon.ne</t>
+  </si>
+  <si>
+    <t>Stageman</t>
+  </si>
+  <si>
+    <t>Horaires, Bar public, Bar loges</t>
+  </si>
+  <si>
+    <t>Rieger</t>
+  </si>
+  <si>
+    <t>Maya</t>
+  </si>
+  <si>
+    <t>Artiste</t>
   </si>
 </sst>
 </file>
@@ -1056,16 +1071,16 @@
         </row>
         <row r="65">
           <cell r="B65" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="E65" t="str">
-            <v>Delassus</v>
+            <v>Ménard</v>
           </cell>
           <cell r="F65" t="str">
-            <v>Frank</v>
+            <v>Mireille</v>
           </cell>
           <cell r="L65" t="str">
-            <v>Artiste</v>
+            <v>Staff</v>
           </cell>
         </row>
         <row r="66">
@@ -1073,10 +1088,10 @@
             <v>0</v>
           </cell>
           <cell r="E66" t="str">
-            <v>Rieger</v>
+            <v>Delassus</v>
           </cell>
           <cell r="F66" t="str">
-            <v>Maya</v>
+            <v>Frank</v>
           </cell>
           <cell r="L66" t="str">
             <v>Artiste</v>
@@ -1087,10 +1102,10 @@
             <v>0</v>
           </cell>
           <cell r="E67" t="str">
-            <v>Michel</v>
+            <v>Rieger</v>
           </cell>
           <cell r="F67" t="str">
-            <v>Mehdi</v>
+            <v>Maya</v>
           </cell>
           <cell r="L67" t="str">
             <v>Artiste</v>
@@ -1101,10 +1116,10 @@
             <v>0</v>
           </cell>
           <cell r="E68" t="str">
-            <v>Ménard</v>
+            <v>Michel</v>
           </cell>
           <cell r="F68" t="str">
-            <v>Mireille</v>
+            <v>Mehdi</v>
           </cell>
           <cell r="L68" t="str">
             <v>Artiste</v>
@@ -1115,10 +1130,10 @@
             <v>0</v>
           </cell>
           <cell r="E69" t="str">
-            <v>Goumaz</v>
+            <v>Pieper</v>
           </cell>
           <cell r="F69" t="str">
-            <v>Alexandre</v>
+            <v>Giulia</v>
           </cell>
         </row>
         <row r="70">
@@ -1126,10 +1141,10 @@
             <v>0</v>
           </cell>
           <cell r="E70" t="str">
-            <v>Pieper</v>
+            <v>Durand</v>
           </cell>
           <cell r="F70" t="str">
-            <v>Giulia</v>
+            <v>Isidore</v>
           </cell>
         </row>
         <row r="71">
@@ -1137,29 +1152,29 @@
             <v>0</v>
           </cell>
           <cell r="E71" t="str">
-            <v>Durand</v>
+            <v>Lemay</v>
           </cell>
           <cell r="F71" t="str">
-            <v>Isidore</v>
+            <v>Mae</v>
           </cell>
         </row>
         <row r="72">
           <cell r="B72" t="b">
             <v>0</v>
           </cell>
-          <cell r="E72" t="str">
-            <v>Lemay</v>
-          </cell>
           <cell r="F72" t="str">
-            <v>Mae</v>
+            <v>Michelle-Evy</v>
           </cell>
         </row>
         <row r="73">
           <cell r="B73" t="b">
             <v>0</v>
           </cell>
+          <cell r="E73" t="str">
+            <v>Bonay</v>
+          </cell>
           <cell r="F73" t="str">
-            <v>Michelle-Evy</v>
+            <v>Paul</v>
           </cell>
         </row>
         <row r="74">
@@ -1167,10 +1182,10 @@
             <v>0</v>
           </cell>
           <cell r="E74" t="str">
-            <v>Bonay</v>
+            <v>Lagier</v>
           </cell>
           <cell r="F74" t="str">
-            <v>Paul</v>
+            <v>Tician</v>
           </cell>
         </row>
         <row r="75">
@@ -1178,10 +1193,10 @@
             <v>0</v>
           </cell>
           <cell r="E75" t="str">
-            <v>Lagier</v>
+            <v>Carrière</v>
           </cell>
           <cell r="F75" t="str">
-            <v>Tician</v>
+            <v>Zellie</v>
           </cell>
         </row>
         <row r="76">
@@ -1189,10 +1204,10 @@
             <v>0</v>
           </cell>
           <cell r="E76" t="str">
-            <v>Carrière</v>
+            <v>Goumaz</v>
           </cell>
           <cell r="F76" t="str">
-            <v>Zellie</v>
+            <v>Alexandre</v>
           </cell>
         </row>
         <row r="77">
@@ -1238,9 +1253,6 @@
           <cell r="F80" t="str">
             <v>David</v>
           </cell>
-          <cell r="L80" t="str">
-            <v>Staff</v>
-          </cell>
         </row>
         <row r="81">
           <cell r="B81" t="b">
@@ -1394,30 +1406,30 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13"/>
-      <sheetData sheetId="14"/>
-      <sheetData sheetId="15"/>
-      <sheetData sheetId="16"/>
-      <sheetData sheetId="17"/>
-      <sheetData sheetId="18"/>
-      <sheetData sheetId="19"/>
-      <sheetData sheetId="20"/>
-      <sheetData sheetId="21"/>
-      <sheetData sheetId="22"/>
-      <sheetData sheetId="23"/>
-      <sheetData sheetId="24"/>
+      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="2" refreshError="1"/>
+      <sheetData sheetId="3" refreshError="1"/>
+      <sheetData sheetId="4" refreshError="1"/>
+      <sheetData sheetId="5" refreshError="1"/>
+      <sheetData sheetId="6" refreshError="1"/>
+      <sheetData sheetId="7" refreshError="1"/>
+      <sheetData sheetId="8" refreshError="1"/>
+      <sheetData sheetId="9" refreshError="1"/>
+      <sheetData sheetId="10" refreshError="1"/>
+      <sheetData sheetId="11" refreshError="1"/>
+      <sheetData sheetId="12" refreshError="1"/>
+      <sheetData sheetId="13" refreshError="1"/>
+      <sheetData sheetId="14" refreshError="1"/>
+      <sheetData sheetId="15" refreshError="1"/>
+      <sheetData sheetId="16" refreshError="1"/>
+      <sheetData sheetId="17" refreshError="1"/>
+      <sheetData sheetId="18" refreshError="1"/>
+      <sheetData sheetId="19" refreshError="1"/>
+      <sheetData sheetId="20" refreshError="1"/>
+      <sheetData sheetId="21" refreshError="1"/>
+      <sheetData sheetId="22" refreshError="1"/>
+      <sheetData sheetId="23" refreshError="1"/>
+      <sheetData sheetId="24" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -1708,7 +1720,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D62"/>
+  <dimension ref="A1:D64"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="3" width="14.4609375" customWidth="1"/>
@@ -1731,14 +1743,14 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="str" cm="1">
-        <f t="array" ref="A2:B62">_xlfn._xlws.FILTER('[1]Bénévoles 2026 V2'!$E:$F,'[1]Bénévoles 2026 V2'!$B:$B=TRUE)</f>
+        <f t="array" ref="A2:B63">_xlfn._xlws.FILTER('[1]Bénévoles 2026 V2'!$E:$F,'[1]Bénévoles 2026 V2'!$B:$B=TRUE)</f>
         <v>Bouvet</v>
       </c>
       <c r="B2" t="str">
         <v>Agathe</v>
       </c>
       <c r="C2" t="str" cm="1">
-        <f t="array" ref="C2:C62">_xlfn._xlws.FILTER('[1]Bénévoles 2026 V2'!$L:$L,'[1]Bénévoles 2026 V2'!$B:$B=TRUE)</f>
+        <f t="array" ref="C2:C63">_xlfn._xlws.FILTER('[1]Bénévoles 2026 V2'!$L:$L,'[1]Bénévoles 2026 V2'!$B:$B=TRUE)</f>
         <v>Junior.e</v>
       </c>
       <c r="D2" t="s">
@@ -1924,7 +1936,7 @@
         <v>Staff</v>
       </c>
       <c r="D15" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.4">
@@ -1980,7 +1992,7 @@
         <v>Staff</v>
       </c>
       <c r="D19" t="s">
-        <v>2</v>
+        <v>11</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.4">
@@ -2008,7 +2020,7 @@
         <v>Staff</v>
       </c>
       <c r="D21" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.4">
@@ -2036,7 +2048,7 @@
         <v>Adjoint.e</v>
       </c>
       <c r="D23" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.4">
@@ -2078,7 +2090,7 @@
         <v>Staff</v>
       </c>
       <c r="D26" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.4">
@@ -2190,7 +2202,7 @@
         <v>Adjoint.e</v>
       </c>
       <c r="D34" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.4">
@@ -2246,7 +2258,7 @@
         <v>Adjoint.e</v>
       </c>
       <c r="D38" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.4">
@@ -2260,7 +2272,7 @@
         <v>Staff</v>
       </c>
       <c r="D39" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.4">
@@ -2302,7 +2314,7 @@
         <v>Staff</v>
       </c>
       <c r="D42" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.4">
@@ -2316,7 +2328,7 @@
         <v>Staff</v>
       </c>
       <c r="D43" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.4">
@@ -2413,9 +2425,6 @@
       <c r="C50" t="str">
         <v>COF</v>
       </c>
-      <c r="D50" t="s">
-        <v>2</v>
-      </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A51" t="str">
@@ -2483,9 +2492,6 @@
       <c r="C55" t="str">
         <v>COF</v>
       </c>
-      <c r="D55" t="s">
-        <v>2</v>
-      </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A56" t="str">
@@ -2582,6 +2588,34 @@
         <v>Staff</v>
       </c>
       <c r="D62" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A63" t="str">
+        <v>Ménard</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Mireille</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Staff</v>
+      </c>
+      <c r="D63" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A64" t="s">
+        <v>12</v>
+      </c>
+      <c r="B64" t="s">
+        <v>13</v>
+      </c>
+      <c r="C64" t="s">
+        <v>14</v>
+      </c>
+      <c r="D64" t="s">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Toward a web-based application. Done some cosmetics and introduction
</commit_message>
<xml_diff>
--- a/data/personnes.xlsx
+++ b/data/personnes.xlsx
@@ -2,23 +2,24 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sschies1\_code\1.09_VScode\06_VoeuxConcerts\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9FE3BF7-536A-4DFD-BACE-E02E255DAA87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5CABD82-6FBA-4056-8295-0FEED94ED606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25490" yWindow="1480" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Personnes" sheetId="1" r:id="rId1"/>
+    <sheet name="LOOKUP" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId2"/>
+    <externalReference r:id="rId3"/>
   </externalReferences>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterate="1" iterateCount="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -58,15 +59,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="16">
   <si>
     <t>Nom</t>
   </si>
   <si>
     <t>Capacités</t>
-  </si>
-  <si>
-    <t>Tous</t>
   </si>
   <si>
     <t>Prénom</t>
@@ -104,6 +102,12 @@
   <si>
     <t>Artiste</t>
   </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>FREEZE!</t>
+  </si>
 </sst>
 </file>
 
@@ -126,12 +130,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -146,14 +156,115 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="13">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -164,6 +275,172 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>12700</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="TextBox 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F0629EF2-86D8-4E80-8BBB-7F41216EC15F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5924550" y="184150"/>
+          <a:ext cx="3282950" cy="2762250"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="1" u="sng"/>
+            <a:t>Personnes &amp;</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="1" u="sng" baseline="0"/>
+            <a:t> capacités</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="171450" indent="-171450">
+            <a:buFont typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            <a:buChar char="•"/>
+          </a:pPr>
+          <a:endParaRPr lang="en-GB" sz="1100" baseline="0"/>
+        </a:p>
+        <a:p>
+          <a:pPr marL="171450" indent="-171450">
+            <a:buFont typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            <a:buChar char="•"/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" baseline="0"/>
+            <a:t>Cette liste est une copie de "BENEVOLES26.xlsx"</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="171450" indent="-171450">
+            <a:buFont typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            <a:buChar char="•"/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" baseline="0"/>
+            <a:t>Il est possible d'ajouter en fin de liste des noms supplémentaires</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="171450" indent="-171450">
+            <a:buFont typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            <a:buChar char="•"/>
+          </a:pPr>
+          <a:endParaRPr lang="en-GB" sz="1100" baseline="0"/>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" indent="0">
+            <a:buFont typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            <a:buNone/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" b="1"/>
+            <a:t>Règles</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" b="1" baseline="0"/>
+            <a:t> pour les capacités :</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="171450" indent="-171450">
+            <a:buFont typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            <a:buChar char="•"/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100"/>
+            <a:t>Une case vide ou comprenant</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" baseline="0"/>
+            <a:t> "Tous", "Toutes" ou "*" signifie que la personne peut tout faire</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="171450" indent="-171450">
+            <a:buFont typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            <a:buChar char="•"/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" baseline="0"/>
+            <a:t>Une personne avec une seule capacité n'est pas intégrée dans le solveur; elle s'auto-gère (p.ex. "Bourdon.ne" ou "Accueil")</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="171450" indent="-171450">
+            <a:buFont typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            <a:buChar char="•"/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" baseline="0"/>
+            <a:t>Entrer les capacités de chacun.e séparées par une virgule. </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" b="1" baseline="0"/>
+            <a:t>Attention à l'orthographe!</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-GB" sz="1100" b="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1406,33 +1683,50 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
-      <sheetData sheetId="5" refreshError="1"/>
-      <sheetData sheetId="6" refreshError="1"/>
-      <sheetData sheetId="7" refreshError="1"/>
-      <sheetData sheetId="8" refreshError="1"/>
-      <sheetData sheetId="9" refreshError="1"/>
-      <sheetData sheetId="10" refreshError="1"/>
-      <sheetData sheetId="11" refreshError="1"/>
-      <sheetData sheetId="12" refreshError="1"/>
-      <sheetData sheetId="13" refreshError="1"/>
-      <sheetData sheetId="14" refreshError="1"/>
-      <sheetData sheetId="15" refreshError="1"/>
-      <sheetData sheetId="16" refreshError="1"/>
-      <sheetData sheetId="17" refreshError="1"/>
-      <sheetData sheetId="18" refreshError="1"/>
-      <sheetData sheetId="19" refreshError="1"/>
-      <sheetData sheetId="20" refreshError="1"/>
-      <sheetData sheetId="21" refreshError="1"/>
-      <sheetData sheetId="22" refreshError="1"/>
-      <sheetData sheetId="23" refreshError="1"/>
-      <sheetData sheetId="24" refreshError="1"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
+      <sheetData sheetId="8"/>
+      <sheetData sheetId="9"/>
+      <sheetData sheetId="10"/>
+      <sheetData sheetId="11"/>
+      <sheetData sheetId="12"/>
+      <sheetData sheetId="13"/>
+      <sheetData sheetId="14"/>
+      <sheetData sheetId="15"/>
+      <sheetData sheetId="16"/>
+      <sheetData sheetId="17"/>
+      <sheetData sheetId="18"/>
+      <sheetData sheetId="19"/>
+      <sheetData sheetId="20"/>
+      <sheetData sheetId="21"/>
+      <sheetData sheetId="22"/>
+      <sheetData sheetId="23"/>
+      <sheetData sheetId="24"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
+</file>
+
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <bag type="Checkbox"/>
+  <bag type="XFControls">
+    <bagId k="CellControl">0</bagId>
+  </bag>
+  <bag type="XFComplement">
+    <bagId k="XFControls">1</bagId>
+  </bag>
+  <bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+</FeaturePropertyBags>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1720,11 +2014,1143 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr codeName="Sheet1"/>
+  <dimension ref="A1:L64"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="3" width="14.4609375" customWidth="1"/>
+    <col min="4" max="4" width="40" customWidth="1"/>
+    <col min="5" max="5" width="4.23046875" customWidth="1"/>
+    <col min="11" max="11" width="4" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="A2" t="str">
+        <f>IF($L$3,A2,LOOKUP!A2)</f>
+        <v>Bouvet</v>
+      </c>
+      <c r="B2" t="str">
+        <f>IF($L$3,B2,LOOKUP!B2)</f>
+        <v>Agathe</v>
+      </c>
+      <c r="C2" t="str">
+        <f>IF($L$3,C2,LOOKUP!C2)</f>
+        <v>Junior.e</v>
+      </c>
+      <c r="D2" t="s">
+        <v>14</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="A3" t="str">
+        <f>IF($L$3,A3,LOOKUP!A3)</f>
+        <v>Bulka</v>
+      </c>
+      <c r="B3" t="str">
+        <f>IF($L$3,B3,LOOKUP!B3)</f>
+        <v>Alegria Lily</v>
+      </c>
+      <c r="C3" t="str">
+        <f>IF($L$3,C3,LOOKUP!C3)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D3" t="s">
+        <v>14</v>
+      </c>
+      <c r="L3" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="A4" t="str">
+        <f>IF($L$3,A4,LOOKUP!A4)</f>
+        <v>Bastian</v>
+      </c>
+      <c r="B4" t="str">
+        <f>IF($L$3,B4,LOOKUP!B4)</f>
+        <v>Alexandra</v>
+      </c>
+      <c r="C4" t="str">
+        <f>IF($L$3,C4,LOOKUP!C4)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="A5" t="str">
+        <f>IF($L$3,A5,LOOKUP!A5)</f>
+        <v>L'Horset</v>
+      </c>
+      <c r="B5" t="str">
+        <f>IF($L$3,B5,LOOKUP!B5)</f>
+        <v>Alice</v>
+      </c>
+      <c r="C5" t="str">
+        <f>IF($L$3,C5,LOOKUP!C5)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="A6" t="str">
+        <f>IF($L$3,A6,LOOKUP!A6)</f>
+        <v>Ledru</v>
+      </c>
+      <c r="B6" t="str">
+        <f>IF($L$3,B6,LOOKUP!B6)</f>
+        <v>Analou</v>
+      </c>
+      <c r="C6" t="str">
+        <f>IF($L$3,C6,LOOKUP!C6)</f>
+        <v>Junior.e</v>
+      </c>
+      <c r="D6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="A7" t="str">
+        <f>IF($L$3,A7,LOOKUP!A7)</f>
+        <v>Mallet</v>
+      </c>
+      <c r="B7" t="str">
+        <f>IF($L$3,B7,LOOKUP!B7)</f>
+        <v>Anna</v>
+      </c>
+      <c r="C7" t="str">
+        <f>IF($L$3,C7,LOOKUP!C7)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="A8" t="str">
+        <f>IF($L$3,A8,LOOKUP!A8)</f>
+        <v>Malric</v>
+      </c>
+      <c r="B8" t="str">
+        <f>IF($L$3,B8,LOOKUP!B8)</f>
+        <v>Annouk</v>
+      </c>
+      <c r="C8" t="str">
+        <f>IF($L$3,C8,LOOKUP!C8)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="A9" t="str">
+        <f>IF($L$3,A9,LOOKUP!A9)</f>
+        <v>Noël</v>
+      </c>
+      <c r="B9" t="str">
+        <f>IF($L$3,B9,LOOKUP!B9)</f>
+        <v>Antonin</v>
+      </c>
+      <c r="C9" t="str">
+        <f>IF($L$3,C9,LOOKUP!C9)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="A10" t="str">
+        <f>IF($L$3,A10,LOOKUP!A10)</f>
+        <v>Tessier</v>
+      </c>
+      <c r="B10" t="str">
+        <f>IF($L$3,B10,LOOKUP!B10)</f>
+        <v>Arsène</v>
+      </c>
+      <c r="C10" t="str">
+        <f>IF($L$3,C10,LOOKUP!C10)</f>
+        <v>Junior.e</v>
+      </c>
+      <c r="D10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="A11" t="str">
+        <f>IF($L$3,A11,LOOKUP!A11)</f>
+        <v>Uldry</v>
+      </c>
+      <c r="B11" t="str">
+        <f>IF($L$3,B11,LOOKUP!B11)</f>
+        <v>Arthur</v>
+      </c>
+      <c r="C11" t="str">
+        <f>IF($L$3,C11,LOOKUP!C11)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D11" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="A12" t="str">
+        <f>IF($L$3,A12,LOOKUP!A12)</f>
+        <v>Marchand</v>
+      </c>
+      <c r="B12" t="str">
+        <f>IF($L$3,B12,LOOKUP!B12)</f>
+        <v>Athénaé</v>
+      </c>
+      <c r="C12" t="str">
+        <f>IF($L$3,C12,LOOKUP!C12)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D12" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="A13" t="str">
+        <f>IF($L$3,A13,LOOKUP!A13)</f>
+        <v>Magerand</v>
+      </c>
+      <c r="B13" t="str">
+        <f>IF($L$3,B13,LOOKUP!B13)</f>
+        <v>Auxence</v>
+      </c>
+      <c r="C13" t="str">
+        <f>IF($L$3,C13,LOOKUP!C13)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="A14" t="str">
+        <f>IF($L$3,A14,LOOKUP!A14)</f>
+        <v>Baruch</v>
+      </c>
+      <c r="B14" t="str">
+        <f>IF($L$3,B14,LOOKUP!B14)</f>
+        <v>Ava</v>
+      </c>
+      <c r="C14" t="str">
+        <f>IF($L$3,C14,LOOKUP!C14)</f>
+        <v>Junior.e</v>
+      </c>
+      <c r="D14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="A15" t="str">
+        <f>IF($L$3,A15,LOOKUP!A15)</f>
+        <v>Detrain</v>
+      </c>
+      <c r="B15" t="str">
+        <f>IF($L$3,B15,LOOKUP!B15)</f>
+        <v>Benoît</v>
+      </c>
+      <c r="C15" t="str">
+        <f>IF($L$3,C15,LOOKUP!C15)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="A16" t="str">
+        <f>IF($L$3,A16,LOOKUP!A16)</f>
+        <v>Meige</v>
+      </c>
+      <c r="B16" t="str">
+        <f>IF($L$3,B16,LOOKUP!B16)</f>
+        <v>Corentin</v>
+      </c>
+      <c r="C16" t="str">
+        <f>IF($L$3,C16,LOOKUP!C16)</f>
+        <v>Adjoint.e</v>
+      </c>
+      <c r="D16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A17" t="str">
+        <f>IF($L$3,A17,LOOKUP!A17)</f>
+        <v>De Filippo</v>
+      </c>
+      <c r="B17" t="str">
+        <f>IF($L$3,B17,LOOKUP!B17)</f>
+        <v>Emma</v>
+      </c>
+      <c r="C17" t="str">
+        <f>IF($L$3,C17,LOOKUP!C17)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D17" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A18" t="str">
+        <f>IF($L$3,A18,LOOKUP!A18)</f>
+        <v>Maître</v>
+      </c>
+      <c r="B18" t="str">
+        <f>IF($L$3,B18,LOOKUP!B18)</f>
+        <v>Enzo</v>
+      </c>
+      <c r="C18" t="str">
+        <f>IF($L$3,C18,LOOKUP!C18)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D18" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A19" t="str">
+        <f>IF($L$3,A19,LOOKUP!A19)</f>
+        <v>Prouvost</v>
+      </c>
+      <c r="B19" t="str">
+        <f>IF($L$3,B19,LOOKUP!B19)</f>
+        <v>Eugénie</v>
+      </c>
+      <c r="C19" t="str">
+        <f>IF($L$3,C19,LOOKUP!C19)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D19" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A20" t="str">
+        <f>IF($L$3,A20,LOOKUP!A20)</f>
+        <v xml:space="preserve">Rakotonandrasana </v>
+      </c>
+      <c r="B20" t="str">
+        <f>IF($L$3,B20,LOOKUP!B20)</f>
+        <v>Iris</v>
+      </c>
+      <c r="C20" t="str">
+        <f>IF($L$3,C20,LOOKUP!C20)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D20" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A21" t="str">
+        <f>IF($L$3,A21,LOOKUP!A21)</f>
+        <v>Bürgisser</v>
+      </c>
+      <c r="B21" t="str">
+        <f>IF($L$3,B21,LOOKUP!B21)</f>
+        <v>Jamilah</v>
+      </c>
+      <c r="C21" t="str">
+        <f>IF($L$3,C21,LOOKUP!C21)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D21" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A22" t="str">
+        <f>IF($L$3,A22,LOOKUP!A22)</f>
+        <v>Ruscio</v>
+      </c>
+      <c r="B22" t="str">
+        <f>IF($L$3,B22,LOOKUP!B22)</f>
+        <v>Jolan</v>
+      </c>
+      <c r="C22" t="str">
+        <f>IF($L$3,C22,LOOKUP!C22)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D22" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A23" t="str">
+        <f>IF($L$3,A23,LOOKUP!A23)</f>
+        <v>Wuilloud</v>
+      </c>
+      <c r="B23" t="str">
+        <f>IF($L$3,B23,LOOKUP!B23)</f>
+        <v xml:space="preserve">Jonas </v>
+      </c>
+      <c r="C23" t="str">
+        <f>IF($L$3,C23,LOOKUP!C23)</f>
+        <v>Adjoint.e</v>
+      </c>
+      <c r="D23" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A24" t="str">
+        <f>IF($L$3,A24,LOOKUP!A24)</f>
+        <v>Pirolley</v>
+      </c>
+      <c r="B24" t="str">
+        <f>IF($L$3,B24,LOOKUP!B24)</f>
+        <v>Jules</v>
+      </c>
+      <c r="C24" t="str">
+        <f>IF($L$3,C24,LOOKUP!C24)</f>
+        <v>Junior.e</v>
+      </c>
+      <c r="D24" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A25" t="str">
+        <f>IF($L$3,A25,LOOKUP!A25)</f>
+        <v>Chavaillaz</v>
+      </c>
+      <c r="B25" t="str">
+        <f>IF($L$3,B25,LOOKUP!B25)</f>
+        <v>Julie</v>
+      </c>
+      <c r="C25" t="str">
+        <f>IF($L$3,C25,LOOKUP!C25)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D25" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A26" t="str">
+        <f>IF($L$3,A26,LOOKUP!A26)</f>
+        <v>Oeschger</v>
+      </c>
+      <c r="B26" t="str">
+        <f>IF($L$3,B26,LOOKUP!B26)</f>
+        <v>Kristel</v>
+      </c>
+      <c r="C26" t="str">
+        <f>IF($L$3,C26,LOOKUP!C26)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D26" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A27" t="str">
+        <f>IF($L$3,A27,LOOKUP!A27)</f>
+        <v>Baltzinger</v>
+      </c>
+      <c r="B27" t="str">
+        <f>IF($L$3,B27,LOOKUP!B27)</f>
+        <v>Léa</v>
+      </c>
+      <c r="C27" t="str">
+        <f>IF($L$3,C27,LOOKUP!C27)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D27" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A28" t="str">
+        <f>IF($L$3,A28,LOOKUP!A28)</f>
+        <v>Chambaz</v>
+      </c>
+      <c r="B28" t="str">
+        <f>IF($L$3,B28,LOOKUP!B28)</f>
+        <v>Léa</v>
+      </c>
+      <c r="C28" t="str">
+        <f>IF($L$3,C28,LOOKUP!C28)</f>
+        <v>Adjoint.e</v>
+      </c>
+      <c r="D28" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A29" t="str">
+        <f>IF($L$3,A29,LOOKUP!A29)</f>
+        <v>Ledru</v>
+      </c>
+      <c r="B29" t="str">
+        <f>IF($L$3,B29,LOOKUP!B29)</f>
+        <v>Lina-Rosa</v>
+      </c>
+      <c r="C29" t="str">
+        <f>IF($L$3,C29,LOOKUP!C29)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D29" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A30" t="str">
+        <f>IF($L$3,A30,LOOKUP!A30)</f>
+        <v>Jaquet</v>
+      </c>
+      <c r="B30" t="str">
+        <f>IF($L$3,B30,LOOKUP!B30)</f>
+        <v>Lisa</v>
+      </c>
+      <c r="C30" t="str">
+        <f>IF($L$3,C30,LOOKUP!C30)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D30" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A31" t="str">
+        <f>IF($L$3,A31,LOOKUP!A31)</f>
+        <v>Magnin</v>
+      </c>
+      <c r="B31" t="str">
+        <f>IF($L$3,B31,LOOKUP!B31)</f>
+        <v>Lisa</v>
+      </c>
+      <c r="C31" t="str">
+        <f>IF($L$3,C31,LOOKUP!C31)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D31" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A32" t="str">
+        <f>IF($L$3,A32,LOOKUP!A32)</f>
+        <v>Cardis</v>
+      </c>
+      <c r="B32" t="str">
+        <f>IF($L$3,B32,LOOKUP!B32)</f>
+        <v>Louis</v>
+      </c>
+      <c r="C32" t="str">
+        <f>IF($L$3,C32,LOOKUP!C32)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D32" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A33" t="str">
+        <f>IF($L$3,A33,LOOKUP!A33)</f>
+        <v>Post</v>
+      </c>
+      <c r="B33" t="str">
+        <f>IF($L$3,B33,LOOKUP!B33)</f>
+        <v>Louis</v>
+      </c>
+      <c r="C33" t="str">
+        <f>IF($L$3,C33,LOOKUP!C33)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D33" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A34" t="str">
+        <f>IF($L$3,A34,LOOKUP!A34)</f>
+        <v>Blanchard</v>
+      </c>
+      <c r="B34" t="str">
+        <f>IF($L$3,B34,LOOKUP!B34)</f>
+        <v>Louise</v>
+      </c>
+      <c r="C34" t="str">
+        <f>IF($L$3,C34,LOOKUP!C34)</f>
+        <v>Adjoint.e</v>
+      </c>
+      <c r="D34" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A35" t="str">
+        <f>IF($L$3,A35,LOOKUP!A35)</f>
+        <v>Chastroux</v>
+      </c>
+      <c r="B35" t="str">
+        <f>IF($L$3,B35,LOOKUP!B35)</f>
+        <v>Lucas</v>
+      </c>
+      <c r="C35" t="str">
+        <f>IF($L$3,C35,LOOKUP!C35)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D35" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A36" t="str">
+        <f>IF($L$3,A36,LOOKUP!A36)</f>
+        <v>Meyer</v>
+      </c>
+      <c r="B36" t="str">
+        <f>IF($L$3,B36,LOOKUP!B36)</f>
+        <v>Lucie</v>
+      </c>
+      <c r="C36" t="str">
+        <f>IF($L$3,C36,LOOKUP!C36)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D36" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A37" t="str">
+        <f>IF($L$3,A37,LOOKUP!A37)</f>
+        <v>Ménétrey</v>
+      </c>
+      <c r="B37" t="str">
+        <f>IF($L$3,B37,LOOKUP!B37)</f>
+        <v>Maëlan</v>
+      </c>
+      <c r="C37" t="str">
+        <f>IF($L$3,C37,LOOKUP!C37)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D37" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A38" t="str">
+        <f>IF($L$3,A38,LOOKUP!A38)</f>
+        <v>Chambaz</v>
+      </c>
+      <c r="B38" t="str">
+        <f>IF($L$3,B38,LOOKUP!B38)</f>
+        <v>Maëlle</v>
+      </c>
+      <c r="C38" t="str">
+        <f>IF($L$3,C38,LOOKUP!C38)</f>
+        <v>Adjoint.e</v>
+      </c>
+      <c r="D38" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A39" t="str">
+        <f>IF($L$3,A39,LOOKUP!A39)</f>
+        <v>Felix</v>
+      </c>
+      <c r="B39" t="str">
+        <f>IF($L$3,B39,LOOKUP!B39)</f>
+        <v>Marius</v>
+      </c>
+      <c r="C39" t="str">
+        <f>IF($L$3,C39,LOOKUP!C39)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A40" t="str">
+        <f>IF($L$3,A40,LOOKUP!A40)</f>
+        <v>Ledru</v>
+      </c>
+      <c r="B40" t="str">
+        <f>IF($L$3,B40,LOOKUP!B40)</f>
+        <v>Marot</v>
+      </c>
+      <c r="C40" t="str">
+        <f>IF($L$3,C40,LOOKUP!C40)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D40" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A41" t="str">
+        <f>IF($L$3,A41,LOOKUP!A41)</f>
+        <v>Cuinet</v>
+      </c>
+      <c r="B41" t="str">
+        <f>IF($L$3,B41,LOOKUP!B41)</f>
+        <v>Mathis</v>
+      </c>
+      <c r="C41" t="str">
+        <f>IF($L$3,C41,LOOKUP!C41)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D41" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A42" t="str">
+        <f>IF($L$3,A42,LOOKUP!A42)</f>
+        <v>Gavin</v>
+      </c>
+      <c r="B42" t="str">
+        <f>IF($L$3,B42,LOOKUP!B42)</f>
+        <v>Matteo</v>
+      </c>
+      <c r="C42" t="str">
+        <f>IF($L$3,C42,LOOKUP!C42)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D42" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A43" t="str">
+        <f>IF($L$3,A43,LOOKUP!A43)</f>
+        <v>Debray</v>
+      </c>
+      <c r="B43" t="str">
+        <f>IF($L$3,B43,LOOKUP!B43)</f>
+        <v>Maxime</v>
+      </c>
+      <c r="C43" t="str">
+        <f>IF($L$3,C43,LOOKUP!C43)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A44" t="str">
+        <f>IF($L$3,A44,LOOKUP!A44)</f>
+        <v>Corbelli</v>
+      </c>
+      <c r="B44" t="str">
+        <f>IF($L$3,B44,LOOKUP!B44)</f>
+        <v>Maya</v>
+      </c>
+      <c r="C44" t="str">
+        <f>IF($L$3,C44,LOOKUP!C44)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D44" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A45" t="str">
+        <f>IF($L$3,A45,LOOKUP!A45)</f>
+        <v>Pasche</v>
+      </c>
+      <c r="B45" t="str">
+        <f>IF($L$3,B45,LOOKUP!B45)</f>
+        <v>Mickaël</v>
+      </c>
+      <c r="C45" t="str">
+        <f>IF($L$3,C45,LOOKUP!C45)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D45" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A46" t="str">
+        <f>IF($L$3,A46,LOOKUP!A46)</f>
+        <v>Fargues</v>
+      </c>
+      <c r="B46" t="str">
+        <f>IF($L$3,B46,LOOKUP!B46)</f>
+        <v>Morgana</v>
+      </c>
+      <c r="C46" t="str">
+        <f>IF($L$3,C46,LOOKUP!C46)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D46" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A47" t="str">
+        <f>IF($L$3,A47,LOOKUP!A47)</f>
+        <v>Scyboz (Lambelet)</v>
+      </c>
+      <c r="B47" t="str">
+        <f>IF($L$3,B47,LOOKUP!B47)</f>
+        <v>Morgane</v>
+      </c>
+      <c r="C47" t="str">
+        <f>IF($L$3,C47,LOOKUP!C47)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D47" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A48" t="str">
+        <f>IF($L$3,A48,LOOKUP!A48)</f>
+        <v>Koux</v>
+      </c>
+      <c r="B48" t="str">
+        <f>IF($L$3,B48,LOOKUP!B48)</f>
+        <v>Nathalia</v>
+      </c>
+      <c r="C48" t="str">
+        <f>IF($L$3,C48,LOOKUP!C48)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D48" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A49" t="str">
+        <f>IF($L$3,A49,LOOKUP!A49)</f>
+        <v>Cherpillod</v>
+      </c>
+      <c r="B49" t="str">
+        <f>IF($L$3,B49,LOOKUP!B49)</f>
+        <v>Noah</v>
+      </c>
+      <c r="C49" t="str">
+        <f>IF($L$3,C49,LOOKUP!C49)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D49" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A50" t="str">
+        <f>IF($L$3,A50,LOOKUP!A50)</f>
+        <v>Chambaz</v>
+      </c>
+      <c r="B50" t="str">
+        <f>IF($L$3,B50,LOOKUP!B50)</f>
+        <v>Patrick</v>
+      </c>
+      <c r="C50" t="str">
+        <f>IF($L$3,C50,LOOKUP!C50)</f>
+        <v>COF</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A51" t="str">
+        <f>IF($L$3,A51,LOOKUP!A51)</f>
+        <v>Assaoui</v>
+      </c>
+      <c r="B51" t="str">
+        <f>IF($L$3,B51,LOOKUP!B51)</f>
+        <v>Rama</v>
+      </c>
+      <c r="C51" t="str">
+        <f>IF($L$3,C51,LOOKUP!C51)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D51" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A52" t="str">
+        <f>IF($L$3,A52,LOOKUP!A52)</f>
+        <v>Lacroze</v>
+      </c>
+      <c r="B52" t="str">
+        <f>IF($L$3,B52,LOOKUP!B52)</f>
+        <v>Raphaël</v>
+      </c>
+      <c r="C52" t="str">
+        <f>IF($L$3,C52,LOOKUP!C52)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D52" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A53" t="str">
+        <f>IF($L$3,A53,LOOKUP!A53)</f>
+        <v>Neidhart</v>
+      </c>
+      <c r="B53" t="str">
+        <f>IF($L$3,B53,LOOKUP!B53)</f>
+        <v>Raphaëlle</v>
+      </c>
+      <c r="C53" t="str">
+        <f>IF($L$3,C53,LOOKUP!C53)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D53" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A54" t="str">
+        <f>IF($L$3,A54,LOOKUP!A54)</f>
+        <v xml:space="preserve">Lanni </v>
+      </c>
+      <c r="B54" t="str">
+        <f>IF($L$3,B54,LOOKUP!B54)</f>
+        <v>Roxanne</v>
+      </c>
+      <c r="C54" t="str">
+        <f>IF($L$3,C54,LOOKUP!C54)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D54" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A55" t="str">
+        <f>IF($L$3,A55,LOOKUP!A55)</f>
+        <v>Schiesser</v>
+      </c>
+      <c r="B55" t="str">
+        <f>IF($L$3,B55,LOOKUP!B55)</f>
+        <v>Sébastien</v>
+      </c>
+      <c r="C55" t="str">
+        <f>IF($L$3,C55,LOOKUP!C55)</f>
+        <v>COF</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A56" t="str">
+        <f>IF($L$3,A56,LOOKUP!A56)</f>
+        <v>Lambelet</v>
+      </c>
+      <c r="B56" t="str">
+        <f>IF($L$3,B56,LOOKUP!B56)</f>
+        <v>Simon</v>
+      </c>
+      <c r="C56" t="str">
+        <f>IF($L$3,C56,LOOKUP!C56)</f>
+        <v>Adjoint.e</v>
+      </c>
+      <c r="D56" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A57" t="str">
+        <f>IF($L$3,A57,LOOKUP!A57)</f>
+        <v>Cyprien</v>
+      </c>
+      <c r="B57" t="str">
+        <f>IF($L$3,B57,LOOKUP!B57)</f>
+        <v>Theo</v>
+      </c>
+      <c r="C57" t="str">
+        <f>IF($L$3,C57,LOOKUP!C57)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D57" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A58" t="str">
+        <f>IF($L$3,A58,LOOKUP!A58)</f>
+        <v>Clerici</v>
+      </c>
+      <c r="B58" t="str">
+        <f>IF($L$3,B58,LOOKUP!B58)</f>
+        <v>Thibault</v>
+      </c>
+      <c r="C58" t="str">
+        <f>IF($L$3,C58,LOOKUP!C58)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D58" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A59" t="str">
+        <f>IF($L$3,A59,LOOKUP!A59)</f>
+        <v>Ménétrey</v>
+      </c>
+      <c r="B59" t="str">
+        <f>IF($L$3,B59,LOOKUP!B59)</f>
+        <v>Titouan</v>
+      </c>
+      <c r="C59" t="str">
+        <f>IF($L$3,C59,LOOKUP!C59)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D59" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A60" t="str">
+        <f>IF($L$3,A60,LOOKUP!A60)</f>
+        <v>Clerici</v>
+      </c>
+      <c r="B60" t="str">
+        <f>IF($L$3,B60,LOOKUP!B60)</f>
+        <v>Tristan</v>
+      </c>
+      <c r="C60" t="str">
+        <f>IF($L$3,C60,LOOKUP!C60)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D60" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A61" t="str">
+        <f>IF($L$3,A61,LOOKUP!A61)</f>
+        <v>Bally</v>
+      </c>
+      <c r="B61" t="str">
+        <f>IF($L$3,B61,LOOKUP!B61)</f>
+        <v>Yann</v>
+      </c>
+      <c r="C61" t="str">
+        <f>IF($L$3,C61,LOOKUP!C61)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D61" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A62" t="str">
+        <f>IF($L$3,A62,LOOKUP!A62)</f>
+        <v>Ménétrey</v>
+      </c>
+      <c r="B62" t="str">
+        <f>IF($L$3,B62,LOOKUP!B62)</f>
+        <v>Ysatis</v>
+      </c>
+      <c r="C62" t="str">
+        <f>IF($L$3,C62,LOOKUP!C62)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D62" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A63" t="str">
+        <f>IF($L$3,A63,LOOKUP!A63)</f>
+        <v>Ménard</v>
+      </c>
+      <c r="B63" t="str">
+        <f>IF($L$3,B63,LOOKUP!B63)</f>
+        <v>Mireille</v>
+      </c>
+      <c r="C63" t="str">
+        <f>IF($L$3,C63,LOOKUP!C63)</f>
+        <v>Staff</v>
+      </c>
+      <c r="D63" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A64" t="s">
+        <v>11</v>
+      </c>
+      <c r="B64" t="s">
+        <v>12</v>
+      </c>
+      <c r="C64" t="s">
+        <v>13</v>
+      </c>
+      <c r="D64" t="s">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
+  <protectedRanges>
+    <protectedRange sqref="D1:D1048576" name="Capacités"/>
+  </protectedRanges>
+  <conditionalFormatting sqref="A2:XFD67">
+    <cfRule type="expression" dxfId="12" priority="2">
+      <formula>AND(MOD(ROW(),2)=0,$C2="Artiste")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="11" priority="3">
+      <formula>AND(MOD(ROW(),2)=1,$C2="Artiste")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="10" priority="4">
+      <formula>AND(MOD(ROW(),2)=1,$C2="Junior.e")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="9" priority="5">
+      <formula>AND(MOD(ROW(),2)=0,$C2="Junior.e")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="8" priority="6">
+      <formula>AND(MOD(ROW(),2)=0,(OR($C2="Staff",$C2="Adjoint.e",$C2="COF")))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="7" priority="7">
+      <formula>AND(MOD(ROW(),2)=1,(OR($C2="Staff",$C2="Adjoint.e",$C2="COF")))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L2:L3">
+    <cfRule type="expression" dxfId="6" priority="1">
+      <formula>$L$3=TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A39C82D2-536C-412D-A536-F57D990253F2}">
+  <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:D64"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="3" width="14.4609375" customWidth="1"/>
-    <col min="4" max="4" width="31.15234375" customWidth="1"/>
+    <col min="4" max="4" width="40" customWidth="1"/>
+    <col min="5" max="5" width="4.23046875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.4">
@@ -1732,10 +3158,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>3</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>4</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>1</v>
@@ -1754,7 +3180,7 @@
         <v>Junior.e</v>
       </c>
       <c r="D2" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.4">
@@ -1768,7 +3194,7 @@
         <v>Staff</v>
       </c>
       <c r="D3" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.4">
@@ -1782,7 +3208,7 @@
         <v>Staff</v>
       </c>
       <c r="D4" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.4">
@@ -1796,7 +3222,7 @@
         <v>Staff</v>
       </c>
       <c r="D5" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.4">
@@ -1810,7 +3236,7 @@
         <v>Junior.e</v>
       </c>
       <c r="D6" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.4">
@@ -1824,7 +3250,7 @@
         <v>Staff</v>
       </c>
       <c r="D7" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.4">
@@ -1838,7 +3264,7 @@
         <v>Staff</v>
       </c>
       <c r="D8" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.4">
@@ -1852,7 +3278,7 @@
         <v>Staff</v>
       </c>
       <c r="D9" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.4">
@@ -1866,7 +3292,7 @@
         <v>Junior.e</v>
       </c>
       <c r="D10" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.4">
@@ -1880,7 +3306,7 @@
         <v>Staff</v>
       </c>
       <c r="D11" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.4">
@@ -1894,7 +3320,7 @@
         <v>Staff</v>
       </c>
       <c r="D12" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.4">
@@ -1908,7 +3334,7 @@
         <v>Staff</v>
       </c>
       <c r="D13" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.4">
@@ -1922,7 +3348,7 @@
         <v>Junior.e</v>
       </c>
       <c r="D14" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.4">
@@ -1936,7 +3362,7 @@
         <v>Staff</v>
       </c>
       <c r="D15" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.4">
@@ -1950,7 +3376,7 @@
         <v>Adjoint.e</v>
       </c>
       <c r="D16" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.4">
@@ -1964,7 +3390,7 @@
         <v>Staff</v>
       </c>
       <c r="D17" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.4">
@@ -1978,7 +3404,7 @@
         <v>Staff</v>
       </c>
       <c r="D18" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.4">
@@ -1992,7 +3418,7 @@
         <v>Staff</v>
       </c>
       <c r="D19" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.4">
@@ -2006,7 +3432,7 @@
         <v>Staff</v>
       </c>
       <c r="D20" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.4">
@@ -2020,7 +3446,7 @@
         <v>Staff</v>
       </c>
       <c r="D21" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.4">
@@ -2034,7 +3460,7 @@
         <v>Staff</v>
       </c>
       <c r="D22" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.4">
@@ -2048,7 +3474,7 @@
         <v>Adjoint.e</v>
       </c>
       <c r="D23" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.4">
@@ -2062,7 +3488,7 @@
         <v>Junior.e</v>
       </c>
       <c r="D24" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.4">
@@ -2076,7 +3502,7 @@
         <v>Staff</v>
       </c>
       <c r="D25" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.4">
@@ -2090,7 +3516,7 @@
         <v>Staff</v>
       </c>
       <c r="D26" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.4">
@@ -2104,7 +3530,7 @@
         <v>Staff</v>
       </c>
       <c r="D27" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.4">
@@ -2118,7 +3544,7 @@
         <v>Adjoint.e</v>
       </c>
       <c r="D28" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.4">
@@ -2132,7 +3558,7 @@
         <v>Staff</v>
       </c>
       <c r="D29" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.4">
@@ -2146,7 +3572,7 @@
         <v>Staff</v>
       </c>
       <c r="D30" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.4">
@@ -2160,7 +3586,7 @@
         <v>Staff</v>
       </c>
       <c r="D31" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.4">
@@ -2174,7 +3600,7 @@
         <v>Staff</v>
       </c>
       <c r="D32" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.4">
@@ -2188,7 +3614,7 @@
         <v>Staff</v>
       </c>
       <c r="D33" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.4">
@@ -2202,7 +3628,7 @@
         <v>Adjoint.e</v>
       </c>
       <c r="D34" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.4">
@@ -2216,7 +3642,7 @@
         <v>Staff</v>
       </c>
       <c r="D35" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.4">
@@ -2230,7 +3656,7 @@
         <v>Staff</v>
       </c>
       <c r="D36" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.4">
@@ -2244,7 +3670,7 @@
         <v>Staff</v>
       </c>
       <c r="D37" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.4">
@@ -2258,7 +3684,7 @@
         <v>Adjoint.e</v>
       </c>
       <c r="D38" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.4">
@@ -2272,7 +3698,7 @@
         <v>Staff</v>
       </c>
       <c r="D39" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.4">
@@ -2286,7 +3712,7 @@
         <v>Staff</v>
       </c>
       <c r="D40" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.4">
@@ -2300,7 +3726,7 @@
         <v>Staff</v>
       </c>
       <c r="D41" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.4">
@@ -2314,7 +3740,7 @@
         <v>Staff</v>
       </c>
       <c r="D42" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.4">
@@ -2328,7 +3754,7 @@
         <v>Staff</v>
       </c>
       <c r="D43" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.4">
@@ -2342,7 +3768,7 @@
         <v>Staff</v>
       </c>
       <c r="D44" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.4">
@@ -2356,7 +3782,7 @@
         <v>Staff</v>
       </c>
       <c r="D45" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.4">
@@ -2370,7 +3796,7 @@
         <v>Staff</v>
       </c>
       <c r="D46" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.4">
@@ -2384,7 +3810,7 @@
         <v>Staff</v>
       </c>
       <c r="D47" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.4">
@@ -2398,7 +3824,7 @@
         <v>Staff</v>
       </c>
       <c r="D48" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.4">
@@ -2412,7 +3838,7 @@
         <v>Staff</v>
       </c>
       <c r="D49" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.4">
@@ -2437,7 +3863,7 @@
         <v>Staff</v>
       </c>
       <c r="D51" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.4">
@@ -2451,7 +3877,7 @@
         <v>Staff</v>
       </c>
       <c r="D52" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.4">
@@ -2465,7 +3891,7 @@
         <v>Staff</v>
       </c>
       <c r="D53" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.4">
@@ -2479,7 +3905,7 @@
         <v>Staff</v>
       </c>
       <c r="D54" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.4">
@@ -2504,7 +3930,7 @@
         <v>Adjoint.e</v>
       </c>
       <c r="D56" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.4">
@@ -2518,7 +3944,7 @@
         <v>Staff</v>
       </c>
       <c r="D57" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.4">
@@ -2532,7 +3958,7 @@
         <v>Staff</v>
       </c>
       <c r="D58" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.4">
@@ -2546,7 +3972,7 @@
         <v>Staff</v>
       </c>
       <c r="D59" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.4">
@@ -2560,7 +3986,7 @@
         <v>Staff</v>
       </c>
       <c r="D60" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.4">
@@ -2574,7 +4000,7 @@
         <v>Staff</v>
       </c>
       <c r="D61" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.4">
@@ -2588,7 +4014,7 @@
         <v>Staff</v>
       </c>
       <c r="D62" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.4">
@@ -2602,24 +4028,47 @@
         <v>Staff</v>
       </c>
       <c r="D63" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A64" t="s">
+        <v>11</v>
+      </c>
+      <c r="B64" t="s">
         <v>12</v>
       </c>
-      <c r="B64" t="s">
+      <c r="C64" t="s">
         <v>13</v>
       </c>
-      <c r="C64" t="s">
-        <v>14</v>
-      </c>
       <c r="D64" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
+  <protectedRanges>
+    <protectedRange sqref="D1:D1048576" name="Capacités"/>
+  </protectedRanges>
+  <conditionalFormatting sqref="A2:XFD67">
+    <cfRule type="expression" dxfId="5" priority="1">
+      <formula>AND(MOD(ROW(),2)=0,$C2="Artiste")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="4" priority="2">
+      <formula>AND(MOD(ROW(),2)=1,$C2="Artiste")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="3" priority="3">
+      <formula>AND(MOD(ROW(),2)=1,$C2="Junior.e")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="4">
+      <formula>AND(MOD(ROW(),2)=0,$C2="Junior.e")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="5">
+      <formula>AND(MOD(ROW(),2)=0,(OR($C2="Staff",$C2="Adjoint.e",$C2="COF")))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="0" priority="6">
+      <formula>AND(MOD(ROW(),2)=1,(OR($C2="Staff",$C2="Adjoint.e",$C2="COF")))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
- added first real concert wishes - simplified capacités syntax - added alerts for persons missing shifts
</commit_message>
<xml_diff>
--- a/data/personnes.xlsx
+++ b/data/personnes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sschies1\_code\1.09_VScode\06_VoeuxConcerts\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90C4EF20-7514-46B5-9C57-0F46495D3478}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EB880EC-9F97-49CE-9822-A8A55BD9B3E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="129">
   <si>
     <t>Nom</t>
   </si>
@@ -107,6 +107,345 @@
   </si>
   <si>
     <t>FREEZE!</t>
+  </si>
+  <si>
+    <t>Bouvet</t>
+  </si>
+  <si>
+    <t>Agathe</t>
+  </si>
+  <si>
+    <t>Bulka</t>
+  </si>
+  <si>
+    <t>Alegria Lily</t>
+  </si>
+  <si>
+    <t>Bastian</t>
+  </si>
+  <si>
+    <t>Alexandra</t>
+  </si>
+  <si>
+    <t>L'Horset</t>
+  </si>
+  <si>
+    <t>Alice</t>
+  </si>
+  <si>
+    <t>Ledru</t>
+  </si>
+  <si>
+    <t>Analou</t>
+  </si>
+  <si>
+    <t>Mallet</t>
+  </si>
+  <si>
+    <t>Anna</t>
+  </si>
+  <si>
+    <t>Malric</t>
+  </si>
+  <si>
+    <t>Annouk</t>
+  </si>
+  <si>
+    <t>Noël</t>
+  </si>
+  <si>
+    <t>Antonin</t>
+  </si>
+  <si>
+    <t>Tessier</t>
+  </si>
+  <si>
+    <t>Arsène</t>
+  </si>
+  <si>
+    <t>Uldry</t>
+  </si>
+  <si>
+    <t>Arthur</t>
+  </si>
+  <si>
+    <t>Marchand</t>
+  </si>
+  <si>
+    <t>Athénaé</t>
+  </si>
+  <si>
+    <t>Magerand</t>
+  </si>
+  <si>
+    <t>Auxence</t>
+  </si>
+  <si>
+    <t>Baruch</t>
+  </si>
+  <si>
+    <t>Ava</t>
+  </si>
+  <si>
+    <t>Detrain</t>
+  </si>
+  <si>
+    <t>Benoît</t>
+  </si>
+  <si>
+    <t>Meige</t>
+  </si>
+  <si>
+    <t>Corentin</t>
+  </si>
+  <si>
+    <t>De Filippo</t>
+  </si>
+  <si>
+    <t>Emma</t>
+  </si>
+  <si>
+    <t>Maître</t>
+  </si>
+  <si>
+    <t>Enzo</t>
+  </si>
+  <si>
+    <t>Prouvost</t>
+  </si>
+  <si>
+    <t>Eugénie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rakotonandrasana </t>
+  </si>
+  <si>
+    <t>Iris</t>
+  </si>
+  <si>
+    <t>Bürgisser</t>
+  </si>
+  <si>
+    <t>Jamilah</t>
+  </si>
+  <si>
+    <t>Ruscio</t>
+  </si>
+  <si>
+    <t>Jolan</t>
+  </si>
+  <si>
+    <t>Wuilloud</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jonas </t>
+  </si>
+  <si>
+    <t>Pirolley</t>
+  </si>
+  <si>
+    <t>Jules</t>
+  </si>
+  <si>
+    <t>Chavaillaz</t>
+  </si>
+  <si>
+    <t>Julie</t>
+  </si>
+  <si>
+    <t>Oeschger</t>
+  </si>
+  <si>
+    <t>Kristel</t>
+  </si>
+  <si>
+    <t>Baltzinger</t>
+  </si>
+  <si>
+    <t>Léa</t>
+  </si>
+  <si>
+    <t>Chambaz</t>
+  </si>
+  <si>
+    <t>Jaquet</t>
+  </si>
+  <si>
+    <t>Lisa</t>
+  </si>
+  <si>
+    <t>Magnin</t>
+  </si>
+  <si>
+    <t>Cardis</t>
+  </si>
+  <si>
+    <t>Louis</t>
+  </si>
+  <si>
+    <t>Post</t>
+  </si>
+  <si>
+    <t>Blanchard</t>
+  </si>
+  <si>
+    <t>Louise</t>
+  </si>
+  <si>
+    <t>Chastroux</t>
+  </si>
+  <si>
+    <t>Lucas</t>
+  </si>
+  <si>
+    <t>Meyer</t>
+  </si>
+  <si>
+    <t>Lucie</t>
+  </si>
+  <si>
+    <t>Ménétrey</t>
+  </si>
+  <si>
+    <t>Maëlan</t>
+  </si>
+  <si>
+    <t>Maëlle</t>
+  </si>
+  <si>
+    <t>Felix</t>
+  </si>
+  <si>
+    <t>Marius</t>
+  </si>
+  <si>
+    <t>Marot</t>
+  </si>
+  <si>
+    <t>Cuinet</t>
+  </si>
+  <si>
+    <t>Mathis</t>
+  </si>
+  <si>
+    <t>Gavin</t>
+  </si>
+  <si>
+    <t>Matteo</t>
+  </si>
+  <si>
+    <t>Debray</t>
+  </si>
+  <si>
+    <t>Maxime</t>
+  </si>
+  <si>
+    <t>Corbelli</t>
+  </si>
+  <si>
+    <t>Pasche</t>
+  </si>
+  <si>
+    <t>Mickaël</t>
+  </si>
+  <si>
+    <t>Ménard</t>
+  </si>
+  <si>
+    <t>Mireille</t>
+  </si>
+  <si>
+    <t>Fargues</t>
+  </si>
+  <si>
+    <t>Morgana</t>
+  </si>
+  <si>
+    <t>Scyboz (Lambelet)</t>
+  </si>
+  <si>
+    <t>Morgane</t>
+  </si>
+  <si>
+    <t>Koux</t>
+  </si>
+  <si>
+    <t>Nathalia</t>
+  </si>
+  <si>
+    <t>Cherpillod</t>
+  </si>
+  <si>
+    <t>Noah</t>
+  </si>
+  <si>
+    <t>Patrick</t>
+  </si>
+  <si>
+    <t>Assaoui</t>
+  </si>
+  <si>
+    <t>Rama</t>
+  </si>
+  <si>
+    <t>Lacroze</t>
+  </si>
+  <si>
+    <t>Raphaël</t>
+  </si>
+  <si>
+    <t>Neidhart</t>
+  </si>
+  <si>
+    <t>Raphaëlle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lanni </t>
+  </si>
+  <si>
+    <t>Roxanne</t>
+  </si>
+  <si>
+    <t>Schiesser</t>
+  </si>
+  <si>
+    <t>Sébastien</t>
+  </si>
+  <si>
+    <t>Lambelet</t>
+  </si>
+  <si>
+    <t>Simon</t>
+  </si>
+  <si>
+    <t>Cyprien</t>
+  </si>
+  <si>
+    <t>Theo</t>
+  </si>
+  <si>
+    <t>Clerici</t>
+  </si>
+  <si>
+    <t>Thibault</t>
+  </si>
+  <si>
+    <t>Titouan</t>
+  </si>
+  <si>
+    <t>Tristan</t>
+  </si>
+  <si>
+    <t>Bally</t>
+  </si>
+  <si>
+    <t>Yann</t>
+  </si>
+  <si>
+    <t>Ysatis</t>
+  </si>
+  <si>
+    <t>* - bar public</t>
   </si>
 </sst>
 </file>
@@ -217,12 +556,6 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <strike val="0"/>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill>
           <bgColor theme="8" tint="0.39994506668294322"/>
@@ -263,6 +596,12 @@
           <bgColor theme="6" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <color rgb="FFFF0000"/>
+      </font>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -887,10 +1226,10 @@
             <v>1</v>
           </cell>
           <cell r="E31" t="str">
-            <v>Ledru</v>
+            <v>Jaquet</v>
           </cell>
           <cell r="F31" t="str">
-            <v>Lina-Rosa</v>
+            <v>Lisa</v>
           </cell>
           <cell r="L31" t="str">
             <v>Staff</v>
@@ -901,7 +1240,7 @@
             <v>1</v>
           </cell>
           <cell r="E32" t="str">
-            <v>Jaquet</v>
+            <v>Magnin</v>
           </cell>
           <cell r="F32" t="str">
             <v>Lisa</v>
@@ -915,10 +1254,10 @@
             <v>1</v>
           </cell>
           <cell r="E33" t="str">
-            <v>Magnin</v>
+            <v>Cardis</v>
           </cell>
           <cell r="F33" t="str">
-            <v>Lisa</v>
+            <v>Louis</v>
           </cell>
           <cell r="L33" t="str">
             <v>Staff</v>
@@ -929,7 +1268,7 @@
             <v>1</v>
           </cell>
           <cell r="E34" t="str">
-            <v>Cardis</v>
+            <v>Post</v>
           </cell>
           <cell r="F34" t="str">
             <v>Louis</v>
@@ -943,13 +1282,13 @@
             <v>1</v>
           </cell>
           <cell r="E35" t="str">
-            <v>Post</v>
+            <v>Blanchard</v>
           </cell>
           <cell r="F35" t="str">
-            <v>Louis</v>
+            <v>Louise</v>
           </cell>
           <cell r="L35" t="str">
-            <v>Staff</v>
+            <v>Adjoint.e</v>
           </cell>
         </row>
         <row r="36">
@@ -957,13 +1296,13 @@
             <v>1</v>
           </cell>
           <cell r="E36" t="str">
-            <v>Blanchard</v>
+            <v>Chastroux</v>
           </cell>
           <cell r="F36" t="str">
-            <v>Louise</v>
+            <v>Lucas</v>
           </cell>
           <cell r="L36" t="str">
-            <v>Adjoint.e</v>
+            <v>Staff</v>
           </cell>
         </row>
         <row r="37">
@@ -971,10 +1310,10 @@
             <v>1</v>
           </cell>
           <cell r="E37" t="str">
-            <v>Chastroux</v>
+            <v>Meyer</v>
           </cell>
           <cell r="F37" t="str">
-            <v>Lucas</v>
+            <v>Lucie</v>
           </cell>
           <cell r="L37" t="str">
             <v>Staff</v>
@@ -985,10 +1324,10 @@
             <v>1</v>
           </cell>
           <cell r="E38" t="str">
-            <v>Meyer</v>
+            <v>Ménétrey</v>
           </cell>
           <cell r="F38" t="str">
-            <v>Lucie</v>
+            <v>Maëlan</v>
           </cell>
           <cell r="L38" t="str">
             <v>Staff</v>
@@ -999,13 +1338,13 @@
             <v>1</v>
           </cell>
           <cell r="E39" t="str">
-            <v>Ménétrey</v>
+            <v>Chambaz</v>
           </cell>
           <cell r="F39" t="str">
-            <v>Maëlan</v>
+            <v>Maëlle</v>
           </cell>
           <cell r="L39" t="str">
-            <v>Staff</v>
+            <v>Adjoint.e</v>
           </cell>
         </row>
         <row r="40">
@@ -1013,13 +1352,13 @@
             <v>1</v>
           </cell>
           <cell r="E40" t="str">
-            <v>Chambaz</v>
+            <v>Felix</v>
           </cell>
           <cell r="F40" t="str">
-            <v>Maëlle</v>
+            <v>Marius</v>
           </cell>
           <cell r="L40" t="str">
-            <v>Adjoint.e</v>
+            <v>Staff</v>
           </cell>
         </row>
         <row r="41">
@@ -1027,10 +1366,10 @@
             <v>1</v>
           </cell>
           <cell r="E41" t="str">
-            <v>Felix</v>
+            <v>Ledru</v>
           </cell>
           <cell r="F41" t="str">
-            <v>Marius</v>
+            <v>Marot</v>
           </cell>
           <cell r="L41" t="str">
             <v>Staff</v>
@@ -1041,10 +1380,10 @@
             <v>1</v>
           </cell>
           <cell r="E42" t="str">
-            <v>Ledru</v>
+            <v>Cuinet</v>
           </cell>
           <cell r="F42" t="str">
-            <v>Marot</v>
+            <v>Mathis</v>
           </cell>
           <cell r="L42" t="str">
             <v>Staff</v>
@@ -1055,10 +1394,10 @@
             <v>1</v>
           </cell>
           <cell r="E43" t="str">
-            <v>Cuinet</v>
+            <v>Gavin</v>
           </cell>
           <cell r="F43" t="str">
-            <v>Mathis</v>
+            <v>Matteo</v>
           </cell>
           <cell r="L43" t="str">
             <v>Staff</v>
@@ -1069,10 +1408,10 @@
             <v>1</v>
           </cell>
           <cell r="E44" t="str">
-            <v>Gavin</v>
+            <v>Debray</v>
           </cell>
           <cell r="F44" t="str">
-            <v>Matteo</v>
+            <v>Maxime</v>
           </cell>
           <cell r="L44" t="str">
             <v>Staff</v>
@@ -1083,10 +1422,10 @@
             <v>1</v>
           </cell>
           <cell r="E45" t="str">
-            <v>Debray</v>
+            <v>Corbelli</v>
           </cell>
           <cell r="F45" t="str">
-            <v>Maxime</v>
+            <v>Maya</v>
           </cell>
           <cell r="L45" t="str">
             <v>Staff</v>
@@ -1097,10 +1436,10 @@
             <v>1</v>
           </cell>
           <cell r="E46" t="str">
-            <v>Corbelli</v>
+            <v>Pasche</v>
           </cell>
           <cell r="F46" t="str">
-            <v>Maya</v>
+            <v>Mickaël</v>
           </cell>
           <cell r="L46" t="str">
             <v>Staff</v>
@@ -1111,10 +1450,10 @@
             <v>1</v>
           </cell>
           <cell r="E47" t="str">
-            <v>Pasche</v>
+            <v>Ménard</v>
           </cell>
           <cell r="F47" t="str">
-            <v>Mickaël</v>
+            <v>Mireille</v>
           </cell>
           <cell r="L47" t="str">
             <v>Staff</v>
@@ -1362,11 +1701,9 @@
           <cell r="B65" t="b">
             <v>1</v>
           </cell>
-          <cell r="E65" t="str">
-            <v>Ménard</v>
-          </cell>
+          <cell r="E65"/>
           <cell r="F65" t="str">
-            <v>Mireille</v>
+            <v>Andy</v>
           </cell>
           <cell r="L65" t="str">
             <v>Staff</v>
@@ -1544,23 +1881,23 @@
             <v>0</v>
           </cell>
           <cell r="E80" t="str">
-            <v>Gebhardt</v>
+            <v>Aigner</v>
           </cell>
           <cell r="F80" t="str">
             <v>David</v>
           </cell>
-          <cell r="L80"/>
         </row>
         <row r="81">
           <cell r="B81" t="b">
             <v>0</v>
           </cell>
           <cell r="E81" t="str">
-            <v>Aigner</v>
+            <v>Gebhardt</v>
           </cell>
           <cell r="F81" t="str">
             <v>David</v>
           </cell>
+          <cell r="L81"/>
         </row>
         <row r="82">
           <cell r="B82" t="b">
@@ -1589,10 +1926,13 @@
             <v>0</v>
           </cell>
           <cell r="E84" t="str">
-            <v>Bonduel</v>
+            <v>Ledru</v>
           </cell>
           <cell r="F84" t="str">
-            <v>Lola</v>
+            <v>Lina-Rosa</v>
+          </cell>
+          <cell r="L84" t="str">
+            <v>Staff</v>
           </cell>
         </row>
         <row r="85">
@@ -1600,10 +1940,10 @@
             <v>0</v>
           </cell>
           <cell r="E85" t="str">
-            <v>Ledru</v>
+            <v>Bonduel</v>
           </cell>
           <cell r="F85" t="str">
-            <v>Loucas</v>
+            <v>Lola</v>
           </cell>
         </row>
         <row r="86">
@@ -1611,10 +1951,10 @@
             <v>0</v>
           </cell>
           <cell r="E86" t="str">
-            <v>Deschoux</v>
+            <v>Ledru</v>
           </cell>
           <cell r="F86" t="str">
-            <v>Louise</v>
+            <v>Loucas</v>
           </cell>
         </row>
         <row r="87">
@@ -1622,10 +1962,10 @@
             <v>0</v>
           </cell>
           <cell r="E87" t="str">
-            <v>Schlapbach</v>
+            <v>Deschoux</v>
           </cell>
           <cell r="F87" t="str">
-            <v>Naomé</v>
+            <v>Louise</v>
           </cell>
         </row>
         <row r="88">
@@ -1633,10 +1973,10 @@
             <v>0</v>
           </cell>
           <cell r="E88" t="str">
-            <v>Lugeon</v>
+            <v>Schlapbach</v>
           </cell>
           <cell r="F88" t="str">
-            <v>Nicolas</v>
+            <v>Naomé</v>
           </cell>
         </row>
         <row r="89">
@@ -1644,10 +1984,10 @@
             <v>0</v>
           </cell>
           <cell r="E89" t="str">
-            <v>Fogo</v>
+            <v>Lugeon</v>
           </cell>
           <cell r="F89" t="str">
-            <v>Noé</v>
+            <v>Nicolas</v>
           </cell>
         </row>
         <row r="90">
@@ -1655,10 +1995,10 @@
             <v>0</v>
           </cell>
           <cell r="E90" t="str">
-            <v>de Schoulepnikoff</v>
+            <v>Fogo</v>
           </cell>
           <cell r="F90" t="str">
-            <v>Noémie</v>
+            <v>Noé</v>
           </cell>
         </row>
         <row r="91">
@@ -1666,10 +2006,10 @@
             <v>0</v>
           </cell>
           <cell r="E91" t="str">
-            <v>Bouduban</v>
+            <v>de Schoulepnikoff</v>
           </cell>
           <cell r="F91" t="str">
-            <v>Pénélope</v>
+            <v>Noémie</v>
           </cell>
         </row>
         <row r="92">
@@ -1677,38 +2017,49 @@
             <v>0</v>
           </cell>
           <cell r="E92" t="str">
-            <v>Trieu</v>
+            <v>Bouduban</v>
           </cell>
           <cell r="F92" t="str">
-            <v>Raimond</v>
+            <v>Pénélope</v>
           </cell>
         </row>
         <row r="93">
           <cell r="B93" t="b">
             <v>0</v>
           </cell>
-          <cell r="E93"/>
+          <cell r="E93" t="str">
+            <v>Trieu</v>
+          </cell>
           <cell r="F93" t="str">
-            <v>Ramón</v>
-          </cell>
-          <cell r="L93"/>
+            <v>Raimond</v>
+          </cell>
         </row>
         <row r="94">
           <cell r="B94" t="b">
             <v>0</v>
           </cell>
-          <cell r="E94" t="str">
+          <cell r="E94"/>
+          <cell r="F94" t="str">
+            <v>Ramón</v>
+          </cell>
+          <cell r="L94"/>
+        </row>
+        <row r="95">
+          <cell r="B95" t="b">
+            <v>0</v>
+          </cell>
+          <cell r="E95" t="str">
             <v>Aigner</v>
           </cell>
-          <cell r="F94" t="str">
+          <cell r="F95" t="str">
             <v>Robert</v>
           </cell>
         </row>
-        <row r="95">
-          <cell r="B95"/>
-          <cell r="E95"/>
-          <cell r="F95"/>
-          <cell r="L95"/>
+        <row r="96">
+          <cell r="B96"/>
+          <cell r="E96"/>
+          <cell r="F96"/>
+          <cell r="L96"/>
         </row>
       </sheetData>
       <sheetData sheetId="1"/>
@@ -2067,13 +2418,11 @@
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.4">
-      <c r="A2" t="str">
-        <f>IF($L$3,A2,LOOKUP!A2)</f>
-        <v>Bouvet</v>
-      </c>
-      <c r="B2" t="str">
-        <f>IF($L$3,B2,LOOKUP!B2)</f>
-        <v>Agathe</v>
+      <c r="A2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" t="s">
+        <v>17</v>
       </c>
       <c r="C2" t="str">
         <f>IF($L$3,C2,LOOKUP!C2)</f>
@@ -2087,13 +2436,11 @@
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.4">
-      <c r="A3" t="str">
-        <f>IF($L$3,A3,LOOKUP!A3)</f>
-        <v>Bulka</v>
-      </c>
-      <c r="B3" t="str">
-        <f>IF($L$3,B3,LOOKUP!B3)</f>
-        <v>Alegria Lily</v>
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" t="s">
+        <v>19</v>
       </c>
       <c r="C3" t="str">
         <f>IF($L$3,C3,LOOKUP!C3)</f>
@@ -2107,13 +2454,11 @@
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.4">
-      <c r="A4" t="str">
-        <f>IF($L$3,A4,LOOKUP!A4)</f>
-        <v>Bastian</v>
-      </c>
-      <c r="B4" t="str">
-        <f>IF($L$3,B4,LOOKUP!B4)</f>
-        <v>Alexandra</v>
+      <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" t="s">
+        <v>21</v>
       </c>
       <c r="C4" t="str">
         <f>IF($L$3,C4,LOOKUP!C4)</f>
@@ -2124,13 +2469,11 @@
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.4">
-      <c r="A5" t="str">
-        <f>IF($L$3,A5,LOOKUP!A5)</f>
-        <v>L'Horset</v>
-      </c>
-      <c r="B5" t="str">
-        <f>IF($L$3,B5,LOOKUP!B5)</f>
-        <v>Alice</v>
+      <c r="A5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" t="s">
+        <v>23</v>
       </c>
       <c r="C5" t="str">
         <f>IF($L$3,C5,LOOKUP!C5)</f>
@@ -2141,13 +2484,11 @@
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.4">
-      <c r="A6" t="str">
-        <f>IF($L$3,A6,LOOKUP!A6)</f>
-        <v>Ledru</v>
-      </c>
-      <c r="B6" t="str">
-        <f>IF($L$3,B6,LOOKUP!B6)</f>
-        <v>Analou</v>
+      <c r="A6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" t="s">
+        <v>25</v>
       </c>
       <c r="C6" t="str">
         <f>IF($L$3,C6,LOOKUP!C6)</f>
@@ -2158,13 +2499,11 @@
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.4">
-      <c r="A7" t="str">
-        <f>IF($L$3,A7,LOOKUP!A7)</f>
-        <v>Mallet</v>
-      </c>
-      <c r="B7" t="str">
-        <f>IF($L$3,B7,LOOKUP!B7)</f>
-        <v>Anna</v>
+      <c r="A7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" t="s">
+        <v>27</v>
       </c>
       <c r="C7" t="str">
         <f>IF($L$3,C7,LOOKUP!C7)</f>
@@ -2175,13 +2514,11 @@
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.4">
-      <c r="A8" t="str">
-        <f>IF($L$3,A8,LOOKUP!A8)</f>
-        <v>Malric</v>
-      </c>
-      <c r="B8" t="str">
-        <f>IF($L$3,B8,LOOKUP!B8)</f>
-        <v>Annouk</v>
+      <c r="A8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" t="s">
+        <v>29</v>
       </c>
       <c r="C8" t="str">
         <f>IF($L$3,C8,LOOKUP!C8)</f>
@@ -2192,13 +2529,11 @@
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.4">
-      <c r="A9" t="str">
-        <f>IF($L$3,A9,LOOKUP!A9)</f>
-        <v>Noël</v>
-      </c>
-      <c r="B9" t="str">
-        <f>IF($L$3,B9,LOOKUP!B9)</f>
-        <v>Antonin</v>
+      <c r="A9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" t="s">
+        <v>31</v>
       </c>
       <c r="C9" t="str">
         <f>IF($L$3,C9,LOOKUP!C9)</f>
@@ -2209,13 +2544,11 @@
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.4">
-      <c r="A10" t="str">
-        <f>IF($L$3,A10,LOOKUP!A10)</f>
-        <v>Tessier</v>
-      </c>
-      <c r="B10" t="str">
-        <f>IF($L$3,B10,LOOKUP!B10)</f>
-        <v>Arsène</v>
+      <c r="A10" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" t="s">
+        <v>33</v>
       </c>
       <c r="C10" t="str">
         <f>IF($L$3,C10,LOOKUP!C10)</f>
@@ -2226,13 +2559,11 @@
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.4">
-      <c r="A11" t="str">
-        <f>IF($L$3,A11,LOOKUP!A11)</f>
-        <v>Uldry</v>
-      </c>
-      <c r="B11" t="str">
-        <f>IF($L$3,B11,LOOKUP!B11)</f>
-        <v>Arthur</v>
+      <c r="A11" t="s">
+        <v>34</v>
+      </c>
+      <c r="B11" t="s">
+        <v>35</v>
       </c>
       <c r="C11" t="str">
         <f>IF($L$3,C11,LOOKUP!C11)</f>
@@ -2243,13 +2574,11 @@
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.4">
-      <c r="A12" t="str">
-        <f>IF($L$3,A12,LOOKUP!A12)</f>
-        <v>Marchand</v>
-      </c>
-      <c r="B12" t="str">
-        <f>IF($L$3,B12,LOOKUP!B12)</f>
-        <v>Athénaé</v>
+      <c r="A12" t="s">
+        <v>36</v>
+      </c>
+      <c r="B12" t="s">
+        <v>37</v>
       </c>
       <c r="C12" t="str">
         <f>IF($L$3,C12,LOOKUP!C12)</f>
@@ -2260,13 +2589,11 @@
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.4">
-      <c r="A13" t="str">
-        <f>IF($L$3,A13,LOOKUP!A13)</f>
-        <v>Magerand</v>
-      </c>
-      <c r="B13" t="str">
-        <f>IF($L$3,B13,LOOKUP!B13)</f>
-        <v>Auxence</v>
+      <c r="A13" t="s">
+        <v>38</v>
+      </c>
+      <c r="B13" t="s">
+        <v>39</v>
       </c>
       <c r="C13" t="str">
         <f>IF($L$3,C13,LOOKUP!C13)</f>
@@ -2277,13 +2604,11 @@
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.4">
-      <c r="A14" t="str">
-        <f>IF($L$3,A14,LOOKUP!A14)</f>
-        <v>Baruch</v>
-      </c>
-      <c r="B14" t="str">
-        <f>IF($L$3,B14,LOOKUP!B14)</f>
-        <v>Ava</v>
+      <c r="A14" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" t="s">
+        <v>41</v>
       </c>
       <c r="C14" t="str">
         <f>IF($L$3,C14,LOOKUP!C14)</f>
@@ -2294,13 +2619,11 @@
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.4">
-      <c r="A15" t="str">
-        <f>IF($L$3,A15,LOOKUP!A15)</f>
-        <v>Detrain</v>
-      </c>
-      <c r="B15" t="str">
-        <f>IF($L$3,B15,LOOKUP!B15)</f>
-        <v>Benoît</v>
+      <c r="A15" t="s">
+        <v>42</v>
+      </c>
+      <c r="B15" t="s">
+        <v>43</v>
       </c>
       <c r="C15" t="str">
         <f>IF($L$3,C15,LOOKUP!C15)</f>
@@ -2311,13 +2634,11 @@
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.4">
-      <c r="A16" t="str">
-        <f>IF($L$3,A16,LOOKUP!A16)</f>
-        <v>Meige</v>
-      </c>
-      <c r="B16" t="str">
-        <f>IF($L$3,B16,LOOKUP!B16)</f>
-        <v>Corentin</v>
+      <c r="A16" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" t="s">
+        <v>45</v>
       </c>
       <c r="C16" t="str">
         <f>IF($L$3,C16,LOOKUP!C16)</f>
@@ -2328,13 +2649,11 @@
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A17" t="str">
-        <f>IF($L$3,A17,LOOKUP!A17)</f>
-        <v>De Filippo</v>
-      </c>
-      <c r="B17" t="str">
-        <f>IF($L$3,B17,LOOKUP!B17)</f>
-        <v>Emma</v>
+      <c r="A17" t="s">
+        <v>46</v>
+      </c>
+      <c r="B17" t="s">
+        <v>47</v>
       </c>
       <c r="C17" t="str">
         <f>IF($L$3,C17,LOOKUP!C17)</f>
@@ -2345,13 +2664,11 @@
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A18" t="str">
-        <f>IF($L$3,A18,LOOKUP!A18)</f>
-        <v>Maître</v>
-      </c>
-      <c r="B18" t="str">
-        <f>IF($L$3,B18,LOOKUP!B18)</f>
-        <v>Enzo</v>
+      <c r="A18" t="s">
+        <v>48</v>
+      </c>
+      <c r="B18" t="s">
+        <v>49</v>
       </c>
       <c r="C18" t="str">
         <f>IF($L$3,C18,LOOKUP!C18)</f>
@@ -2362,13 +2679,11 @@
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A19" t="str">
-        <f>IF($L$3,A19,LOOKUP!A19)</f>
-        <v>Prouvost</v>
-      </c>
-      <c r="B19" t="str">
-        <f>IF($L$3,B19,LOOKUP!B19)</f>
-        <v>Eugénie</v>
+      <c r="A19" t="s">
+        <v>50</v>
+      </c>
+      <c r="B19" t="s">
+        <v>51</v>
       </c>
       <c r="C19" t="str">
         <f>IF($L$3,C19,LOOKUP!C19)</f>
@@ -2379,13 +2694,11 @@
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A20" t="str">
-        <f>IF($L$3,A20,LOOKUP!A20)</f>
-        <v xml:space="preserve">Rakotonandrasana </v>
-      </c>
-      <c r="B20" t="str">
-        <f>IF($L$3,B20,LOOKUP!B20)</f>
-        <v>Iris</v>
+      <c r="A20" t="s">
+        <v>52</v>
+      </c>
+      <c r="B20" t="s">
+        <v>53</v>
       </c>
       <c r="C20" t="str">
         <f>IF($L$3,C20,LOOKUP!C20)</f>
@@ -2396,13 +2709,11 @@
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A21" t="str">
-        <f>IF($L$3,A21,LOOKUP!A21)</f>
-        <v>Bürgisser</v>
-      </c>
-      <c r="B21" t="str">
-        <f>IF($L$3,B21,LOOKUP!B21)</f>
-        <v>Jamilah</v>
+      <c r="A21" t="s">
+        <v>54</v>
+      </c>
+      <c r="B21" t="s">
+        <v>55</v>
       </c>
       <c r="C21" t="str">
         <f>IF($L$3,C21,LOOKUP!C21)</f>
@@ -2413,13 +2724,11 @@
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A22" t="str">
-        <f>IF($L$3,A22,LOOKUP!A22)</f>
-        <v>Ruscio</v>
-      </c>
-      <c r="B22" t="str">
-        <f>IF($L$3,B22,LOOKUP!B22)</f>
-        <v>Jolan</v>
+      <c r="A22" t="s">
+        <v>56</v>
+      </c>
+      <c r="B22" t="s">
+        <v>57</v>
       </c>
       <c r="C22" t="str">
         <f>IF($L$3,C22,LOOKUP!C22)</f>
@@ -2430,13 +2739,11 @@
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A23" t="str">
-        <f>IF($L$3,A23,LOOKUP!A23)</f>
-        <v>Wuilloud</v>
-      </c>
-      <c r="B23" t="str">
-        <f>IF($L$3,B23,LOOKUP!B23)</f>
-        <v xml:space="preserve">Jonas </v>
+      <c r="A23" t="s">
+        <v>58</v>
+      </c>
+      <c r="B23" t="s">
+        <v>59</v>
       </c>
       <c r="C23" t="str">
         <f>IF($L$3,C23,LOOKUP!C23)</f>
@@ -2447,13 +2754,11 @@
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A24" t="str">
-        <f>IF($L$3,A24,LOOKUP!A24)</f>
-        <v>Pirolley</v>
-      </c>
-      <c r="B24" t="str">
-        <f>IF($L$3,B24,LOOKUP!B24)</f>
-        <v>Jules</v>
+      <c r="A24" t="s">
+        <v>60</v>
+      </c>
+      <c r="B24" t="s">
+        <v>61</v>
       </c>
       <c r="C24" t="str">
         <f>IF($L$3,C24,LOOKUP!C24)</f>
@@ -2464,13 +2769,11 @@
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A25" t="str">
-        <f>IF($L$3,A25,LOOKUP!A25)</f>
-        <v>Chavaillaz</v>
-      </c>
-      <c r="B25" t="str">
-        <f>IF($L$3,B25,LOOKUP!B25)</f>
-        <v>Julie</v>
+      <c r="A25" t="s">
+        <v>62</v>
+      </c>
+      <c r="B25" t="s">
+        <v>63</v>
       </c>
       <c r="C25" t="str">
         <f>IF($L$3,C25,LOOKUP!C25)</f>
@@ -2481,13 +2784,11 @@
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A26" t="str">
-        <f>IF($L$3,A26,LOOKUP!A26)</f>
-        <v>Oeschger</v>
-      </c>
-      <c r="B26" t="str">
-        <f>IF($L$3,B26,LOOKUP!B26)</f>
-        <v>Kristel</v>
+      <c r="A26" t="s">
+        <v>64</v>
+      </c>
+      <c r="B26" t="s">
+        <v>65</v>
       </c>
       <c r="C26" t="str">
         <f>IF($L$3,C26,LOOKUP!C26)</f>
@@ -2498,13 +2799,11 @@
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A27" t="str">
-        <f>IF($L$3,A27,LOOKUP!A27)</f>
-        <v>Baltzinger</v>
-      </c>
-      <c r="B27" t="str">
-        <f>IF($L$3,B27,LOOKUP!B27)</f>
-        <v>Léa</v>
+      <c r="A27" t="s">
+        <v>66</v>
+      </c>
+      <c r="B27" t="s">
+        <v>67</v>
       </c>
       <c r="C27" t="str">
         <f>IF($L$3,C27,LOOKUP!C27)</f>
@@ -2515,13 +2814,11 @@
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A28" t="str">
-        <f>IF($L$3,A28,LOOKUP!A28)</f>
-        <v>Chambaz</v>
-      </c>
-      <c r="B28" t="str">
-        <f>IF($L$3,B28,LOOKUP!B28)</f>
-        <v>Léa</v>
+      <c r="A28" t="s">
+        <v>68</v>
+      </c>
+      <c r="B28" t="s">
+        <v>67</v>
       </c>
       <c r="C28" t="str">
         <f>IF($L$3,C28,LOOKUP!C28)</f>
@@ -2532,13 +2829,11 @@
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A29" t="str">
-        <f>IF($L$3,A29,LOOKUP!A29)</f>
-        <v>Ledru</v>
-      </c>
-      <c r="B29" t="str">
-        <f>IF($L$3,B29,LOOKUP!B29)</f>
-        <v>Lina-Rosa</v>
+      <c r="A29" t="s">
+        <v>69</v>
+      </c>
+      <c r="B29" t="s">
+        <v>70</v>
       </c>
       <c r="C29" t="str">
         <f>IF($L$3,C29,LOOKUP!C29)</f>
@@ -2549,47 +2844,41 @@
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A30" t="str">
-        <f>IF($L$3,A30,LOOKUP!A30)</f>
-        <v>Jaquet</v>
-      </c>
-      <c r="B30" t="str">
-        <f>IF($L$3,B30,LOOKUP!B30)</f>
-        <v>Lisa</v>
+      <c r="A30" t="s">
+        <v>71</v>
+      </c>
+      <c r="B30" t="s">
+        <v>70</v>
       </c>
       <c r="C30" t="str">
         <f>IF($L$3,C30,LOOKUP!C30)</f>
         <v>Staff</v>
       </c>
       <c r="D30" t="s">
-        <v>14</v>
+        <v>4</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A31" t="str">
-        <f>IF($L$3,A31,LOOKUP!A31)</f>
-        <v>Magnin</v>
-      </c>
-      <c r="B31" t="str">
-        <f>IF($L$3,B31,LOOKUP!B31)</f>
-        <v>Lisa</v>
+      <c r="A31" t="s">
+        <v>72</v>
+      </c>
+      <c r="B31" t="s">
+        <v>73</v>
       </c>
       <c r="C31" t="str">
         <f>IF($L$3,C31,LOOKUP!C31)</f>
         <v>Staff</v>
       </c>
       <c r="D31" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A32" t="str">
-        <f>IF($L$3,A32,LOOKUP!A32)</f>
-        <v>Cardis</v>
-      </c>
-      <c r="B32" t="str">
-        <f>IF($L$3,B32,LOOKUP!B32)</f>
-        <v>Louis</v>
+      <c r="A32" t="s">
+        <v>74</v>
+      </c>
+      <c r="B32" t="s">
+        <v>73</v>
       </c>
       <c r="C32" t="str">
         <f>IF($L$3,C32,LOOKUP!C32)</f>
@@ -2600,47 +2889,41 @@
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A33" t="str">
-        <f>IF($L$3,A33,LOOKUP!A33)</f>
-        <v>Post</v>
-      </c>
-      <c r="B33" t="str">
-        <f>IF($L$3,B33,LOOKUP!B33)</f>
-        <v>Louis</v>
+      <c r="A33" t="s">
+        <v>75</v>
+      </c>
+      <c r="B33" t="s">
+        <v>76</v>
       </c>
       <c r="C33" t="str">
         <f>IF($L$3,C33,LOOKUP!C33)</f>
-        <v>Staff</v>
+        <v>Adjoint.e</v>
       </c>
       <c r="D33" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A34" t="str">
-        <f>IF($L$3,A34,LOOKUP!A34)</f>
-        <v>Blanchard</v>
-      </c>
-      <c r="B34" t="str">
-        <f>IF($L$3,B34,LOOKUP!B34)</f>
-        <v>Louise</v>
+      <c r="A34" t="s">
+        <v>77</v>
+      </c>
+      <c r="B34" t="s">
+        <v>78</v>
       </c>
       <c r="C34" t="str">
         <f>IF($L$3,C34,LOOKUP!C34)</f>
-        <v>Adjoint.e</v>
+        <v>Staff</v>
       </c>
       <c r="D34" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A35" t="str">
-        <f>IF($L$3,A35,LOOKUP!A35)</f>
-        <v>Chastroux</v>
-      </c>
-      <c r="B35" t="str">
-        <f>IF($L$3,B35,LOOKUP!B35)</f>
-        <v>Lucas</v>
+      <c r="A35" t="s">
+        <v>79</v>
+      </c>
+      <c r="B35" t="s">
+        <v>80</v>
       </c>
       <c r="C35" t="str">
         <f>IF($L$3,C35,LOOKUP!C35)</f>
@@ -2651,13 +2934,11 @@
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A36" t="str">
-        <f>IF($L$3,A36,LOOKUP!A36)</f>
-        <v>Meyer</v>
-      </c>
-      <c r="B36" t="str">
-        <f>IF($L$3,B36,LOOKUP!B36)</f>
-        <v>Lucie</v>
+      <c r="A36" t="s">
+        <v>81</v>
+      </c>
+      <c r="B36" t="s">
+        <v>82</v>
       </c>
       <c r="C36" t="str">
         <f>IF($L$3,C36,LOOKUP!C36)</f>
@@ -2668,64 +2949,56 @@
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A37" t="str">
-        <f>IF($L$3,A37,LOOKUP!A37)</f>
-        <v>Ménétrey</v>
-      </c>
-      <c r="B37" t="str">
-        <f>IF($L$3,B37,LOOKUP!B37)</f>
-        <v>Maëlan</v>
+      <c r="A37" t="s">
+        <v>68</v>
+      </c>
+      <c r="B37" t="s">
+        <v>83</v>
       </c>
       <c r="C37" t="str">
         <f>IF($L$3,C37,LOOKUP!C37)</f>
-        <v>Staff</v>
+        <v>Adjoint.e</v>
       </c>
       <c r="D37" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A38" t="str">
-        <f>IF($L$3,A38,LOOKUP!A38)</f>
-        <v>Chambaz</v>
-      </c>
-      <c r="B38" t="str">
-        <f>IF($L$3,B38,LOOKUP!B38)</f>
-        <v>Maëlle</v>
+      <c r="A38" t="s">
+        <v>84</v>
+      </c>
+      <c r="B38" t="s">
+        <v>85</v>
       </c>
       <c r="C38" t="str">
         <f>IF($L$3,C38,LOOKUP!C38)</f>
-        <v>Adjoint.e</v>
+        <v>Staff</v>
       </c>
       <c r="D38" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A39" t="str">
-        <f>IF($L$3,A39,LOOKUP!A39)</f>
-        <v>Felix</v>
-      </c>
-      <c r="B39" t="str">
-        <f>IF($L$3,B39,LOOKUP!B39)</f>
-        <v>Marius</v>
+      <c r="A39" t="s">
+        <v>24</v>
+      </c>
+      <c r="B39" t="s">
+        <v>86</v>
       </c>
       <c r="C39" t="str">
         <f>IF($L$3,C39,LOOKUP!C39)</f>
         <v>Staff</v>
       </c>
       <c r="D39" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A40" t="str">
-        <f>IF($L$3,A40,LOOKUP!A40)</f>
-        <v>Ledru</v>
-      </c>
-      <c r="B40" t="str">
-        <f>IF($L$3,B40,LOOKUP!B40)</f>
-        <v>Marot</v>
+      <c r="A40" t="s">
+        <v>87</v>
+      </c>
+      <c r="B40" t="s">
+        <v>88</v>
       </c>
       <c r="C40" t="str">
         <f>IF($L$3,C40,LOOKUP!C40)</f>
@@ -2736,13 +3009,11 @@
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A41" t="str">
-        <f>IF($L$3,A41,LOOKUP!A41)</f>
-        <v>Cuinet</v>
-      </c>
-      <c r="B41" t="str">
-        <f>IF($L$3,B41,LOOKUP!B41)</f>
-        <v>Mathis</v>
+      <c r="A41" t="s">
+        <v>89</v>
+      </c>
+      <c r="B41" t="s">
+        <v>90</v>
       </c>
       <c r="C41" t="str">
         <f>IF($L$3,C41,LOOKUP!C41)</f>
@@ -2753,47 +3024,41 @@
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A42" t="str">
-        <f>IF($L$3,A42,LOOKUP!A42)</f>
-        <v>Gavin</v>
-      </c>
-      <c r="B42" t="str">
-        <f>IF($L$3,B42,LOOKUP!B42)</f>
-        <v>Matteo</v>
+      <c r="A42" t="s">
+        <v>91</v>
+      </c>
+      <c r="B42" t="s">
+        <v>92</v>
       </c>
       <c r="C42" t="str">
         <f>IF($L$3,C42,LOOKUP!C42)</f>
         <v>Staff</v>
       </c>
       <c r="D42" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A43" t="str">
-        <f>IF($L$3,A43,LOOKUP!A43)</f>
-        <v>Debray</v>
-      </c>
-      <c r="B43" t="str">
-        <f>IF($L$3,B43,LOOKUP!B43)</f>
-        <v>Maxime</v>
+      <c r="A43" t="s">
+        <v>93</v>
+      </c>
+      <c r="B43" t="s">
+        <v>12</v>
       </c>
       <c r="C43" t="str">
         <f>IF($L$3,C43,LOOKUP!C43)</f>
         <v>Staff</v>
       </c>
       <c r="D43" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A44" t="str">
-        <f>IF($L$3,A44,LOOKUP!A44)</f>
-        <v>Corbelli</v>
-      </c>
-      <c r="B44" t="str">
-        <f>IF($L$3,B44,LOOKUP!B44)</f>
-        <v>Maya</v>
+      <c r="A44" t="s">
+        <v>94</v>
+      </c>
+      <c r="B44" t="s">
+        <v>95</v>
       </c>
       <c r="C44" t="str">
         <f>IF($L$3,C44,LOOKUP!C44)</f>
@@ -2804,13 +3069,11 @@
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A45" t="str">
-        <f>IF($L$3,A45,LOOKUP!A45)</f>
-        <v>Pasche</v>
-      </c>
-      <c r="B45" t="str">
-        <f>IF($L$3,B45,LOOKUP!B45)</f>
-        <v>Mickaël</v>
+      <c r="A45" t="s">
+        <v>96</v>
+      </c>
+      <c r="B45" t="s">
+        <v>97</v>
       </c>
       <c r="C45" t="str">
         <f>IF($L$3,C45,LOOKUP!C45)</f>
@@ -2821,13 +3084,11 @@
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A46" t="str">
-        <f>IF($L$3,A46,LOOKUP!A46)</f>
-        <v>Fargues</v>
-      </c>
-      <c r="B46" t="str">
-        <f>IF($L$3,B46,LOOKUP!B46)</f>
-        <v>Morgana</v>
+      <c r="A46" t="s">
+        <v>98</v>
+      </c>
+      <c r="B46" t="s">
+        <v>99</v>
       </c>
       <c r="C46" t="str">
         <f>IF($L$3,C46,LOOKUP!C46)</f>
@@ -2838,13 +3099,11 @@
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A47" t="str">
-        <f>IF($L$3,A47,LOOKUP!A47)</f>
-        <v>Scyboz (Lambelet)</v>
-      </c>
-      <c r="B47" t="str">
-        <f>IF($L$3,B47,LOOKUP!B47)</f>
-        <v>Morgane</v>
+      <c r="A47" t="s">
+        <v>100</v>
+      </c>
+      <c r="B47" t="s">
+        <v>101</v>
       </c>
       <c r="C47" t="str">
         <f>IF($L$3,C47,LOOKUP!C47)</f>
@@ -2855,13 +3114,11 @@
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A48" t="str">
-        <f>IF($L$3,A48,LOOKUP!A48)</f>
-        <v>Koux</v>
-      </c>
-      <c r="B48" t="str">
-        <f>IF($L$3,B48,LOOKUP!B48)</f>
-        <v>Nathalia</v>
+      <c r="A48" t="s">
+        <v>102</v>
+      </c>
+      <c r="B48" t="s">
+        <v>103</v>
       </c>
       <c r="C48" t="str">
         <f>IF($L$3,C48,LOOKUP!C48)</f>
@@ -2872,13 +3129,11 @@
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A49" t="str">
-        <f>IF($L$3,A49,LOOKUP!A49)</f>
-        <v>Cherpillod</v>
-      </c>
-      <c r="B49" t="str">
-        <f>IF($L$3,B49,LOOKUP!B49)</f>
-        <v>Noah</v>
+      <c r="A49" t="s">
+        <v>104</v>
+      </c>
+      <c r="B49" t="s">
+        <v>105</v>
       </c>
       <c r="C49" t="str">
         <f>IF($L$3,C49,LOOKUP!C49)</f>
@@ -2889,13 +3144,11 @@
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A50" t="str">
-        <f>IF($L$3,A50,LOOKUP!A50)</f>
-        <v>Chambaz</v>
-      </c>
-      <c r="B50" t="str">
-        <f>IF($L$3,B50,LOOKUP!B50)</f>
-        <v>Patrick</v>
+      <c r="A50" t="s">
+        <v>68</v>
+      </c>
+      <c r="B50" t="s">
+        <v>106</v>
       </c>
       <c r="C50" t="str">
         <f>IF($L$3,C50,LOOKUP!C50)</f>
@@ -2903,30 +3156,26 @@
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A51" t="str">
-        <f>IF($L$3,A51,LOOKUP!A51)</f>
-        <v>Assaoui</v>
-      </c>
-      <c r="B51" t="str">
-        <f>IF($L$3,B51,LOOKUP!B51)</f>
-        <v>Rama</v>
+      <c r="A51" t="s">
+        <v>107</v>
+      </c>
+      <c r="B51" t="s">
+        <v>108</v>
       </c>
       <c r="C51" t="str">
         <f>IF($L$3,C51,LOOKUP!C51)</f>
         <v>Staff</v>
       </c>
       <c r="D51" t="s">
-        <v>14</v>
+        <v>128</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A52" t="str">
-        <f>IF($L$3,A52,LOOKUP!A52)</f>
-        <v>Lacroze</v>
-      </c>
-      <c r="B52" t="str">
-        <f>IF($L$3,B52,LOOKUP!B52)</f>
-        <v>Raphaël</v>
+      <c r="A52" t="s">
+        <v>109</v>
+      </c>
+      <c r="B52" t="s">
+        <v>110</v>
       </c>
       <c r="C52" t="str">
         <f>IF($L$3,C52,LOOKUP!C52)</f>
@@ -2937,13 +3186,11 @@
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A53" t="str">
-        <f>IF($L$3,A53,LOOKUP!A53)</f>
-        <v>Neidhart</v>
-      </c>
-      <c r="B53" t="str">
-        <f>IF($L$3,B53,LOOKUP!B53)</f>
-        <v>Raphaëlle</v>
+      <c r="A53" t="s">
+        <v>111</v>
+      </c>
+      <c r="B53" t="s">
+        <v>112</v>
       </c>
       <c r="C53" t="str">
         <f>IF($L$3,C53,LOOKUP!C53)</f>
@@ -2954,13 +3201,11 @@
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A54" t="str">
-        <f>IF($L$3,A54,LOOKUP!A54)</f>
-        <v xml:space="preserve">Lanni </v>
-      </c>
-      <c r="B54" t="str">
-        <f>IF($L$3,B54,LOOKUP!B54)</f>
-        <v>Roxanne</v>
+      <c r="A54" t="s">
+        <v>113</v>
+      </c>
+      <c r="B54" t="s">
+        <v>114</v>
       </c>
       <c r="C54" t="str">
         <f>IF($L$3,C54,LOOKUP!C54)</f>
@@ -2971,13 +3216,11 @@
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A55" t="str">
-        <f>IF($L$3,A55,LOOKUP!A55)</f>
-        <v>Schiesser</v>
-      </c>
-      <c r="B55" t="str">
-        <f>IF($L$3,B55,LOOKUP!B55)</f>
-        <v>Sébastien</v>
+      <c r="A55" t="s">
+        <v>115</v>
+      </c>
+      <c r="B55" t="s">
+        <v>116</v>
       </c>
       <c r="C55" t="str">
         <f>IF($L$3,C55,LOOKUP!C55)</f>
@@ -2985,13 +3228,11 @@
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A56" t="str">
-        <f>IF($L$3,A56,LOOKUP!A56)</f>
-        <v>Lambelet</v>
-      </c>
-      <c r="B56" t="str">
-        <f>IF($L$3,B56,LOOKUP!B56)</f>
-        <v>Simon</v>
+      <c r="A56" t="s">
+        <v>117</v>
+      </c>
+      <c r="B56" t="s">
+        <v>118</v>
       </c>
       <c r="C56" t="str">
         <f>IF($L$3,C56,LOOKUP!C56)</f>
@@ -3002,13 +3243,11 @@
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A57" t="str">
-        <f>IF($L$3,A57,LOOKUP!A57)</f>
-        <v>Cyprien</v>
-      </c>
-      <c r="B57" t="str">
-        <f>IF($L$3,B57,LOOKUP!B57)</f>
-        <v>Theo</v>
+      <c r="A57" t="s">
+        <v>119</v>
+      </c>
+      <c r="B57" t="s">
+        <v>120</v>
       </c>
       <c r="C57" t="str">
         <f>IF($L$3,C57,LOOKUP!C57)</f>
@@ -3019,13 +3258,11 @@
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A58" t="str">
-        <f>IF($L$3,A58,LOOKUP!A58)</f>
-        <v>Clerici</v>
-      </c>
-      <c r="B58" t="str">
-        <f>IF($L$3,B58,LOOKUP!B58)</f>
-        <v>Thibault</v>
+      <c r="A58" t="s">
+        <v>121</v>
+      </c>
+      <c r="B58" t="s">
+        <v>122</v>
       </c>
       <c r="C58" t="str">
         <f>IF($L$3,C58,LOOKUP!C58)</f>
@@ -3036,13 +3273,11 @@
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A59" t="str">
-        <f>IF($L$3,A59,LOOKUP!A59)</f>
-        <v>Ménétrey</v>
-      </c>
-      <c r="B59" t="str">
-        <f>IF($L$3,B59,LOOKUP!B59)</f>
-        <v>Titouan</v>
+      <c r="A59" t="s">
+        <v>81</v>
+      </c>
+      <c r="B59" t="s">
+        <v>123</v>
       </c>
       <c r="C59" t="str">
         <f>IF($L$3,C59,LOOKUP!C59)</f>
@@ -3053,30 +3288,26 @@
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A60" t="str">
-        <f>IF($L$3,A60,LOOKUP!A60)</f>
-        <v>Clerici</v>
-      </c>
-      <c r="B60" t="str">
-        <f>IF($L$3,B60,LOOKUP!B60)</f>
-        <v>Tristan</v>
+      <c r="A60" t="s">
+        <v>121</v>
+      </c>
+      <c r="B60" t="s">
+        <v>124</v>
       </c>
       <c r="C60" t="str">
         <f>IF($L$3,C60,LOOKUP!C60)</f>
         <v>Staff</v>
       </c>
       <c r="D60" t="s">
-        <v>14</v>
+        <v>128</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A61" t="str">
-        <f>IF($L$3,A61,LOOKUP!A61)</f>
-        <v>Bally</v>
-      </c>
-      <c r="B61" t="str">
-        <f>IF($L$3,B61,LOOKUP!B61)</f>
-        <v>Yann</v>
+      <c r="A61" t="s">
+        <v>125</v>
+      </c>
+      <c r="B61" t="s">
+        <v>126</v>
       </c>
       <c r="C61" t="str">
         <f>IF($L$3,C61,LOOKUP!C61)</f>
@@ -3087,31 +3318,21 @@
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A62" t="str">
-        <f>IF($L$3,A62,LOOKUP!A62)</f>
-        <v>Ménétrey</v>
-      </c>
-      <c r="B62" t="str">
-        <f>IF($L$3,B62,LOOKUP!B62)</f>
-        <v>Ysatis</v>
+      <c r="A62" t="s">
+        <v>81</v>
+      </c>
+      <c r="B62" t="s">
+        <v>127</v>
       </c>
       <c r="C62" t="str">
         <f>IF($L$3,C62,LOOKUP!C62)</f>
         <v>Staff</v>
       </c>
       <c r="D62" t="s">
-        <v>14</v>
+        <v>128</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A63" t="str">
-        <f>IF($L$3,A63,LOOKUP!A63)</f>
-        <v>Ménard</v>
-      </c>
-      <c r="B63" t="str">
-        <f>IF($L$3,B63,LOOKUP!B63)</f>
-        <v>Mireille</v>
-      </c>
       <c r="C63" t="str">
         <f>IF($L$3,C63,LOOKUP!C63)</f>
         <v>Staff</v>
@@ -3121,47 +3342,40 @@
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A64" t="s">
-        <v>11</v>
-      </c>
-      <c r="B64" t="s">
-        <v>12</v>
-      </c>
       <c r="C64" t="s">
         <v>13</v>
       </c>
       <c r="D64" t="s">
-        <v>14</v>
+        <v>128</v>
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <protectedRanges>
     <protectedRange sqref="D1:D1048576" name="Capacités"/>
   </protectedRanges>
+  <conditionalFormatting sqref="L2:L3">
+    <cfRule type="expression" dxfId="12" priority="1">
+      <formula>$L$3=TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A2:XFD67">
-    <cfRule type="expression" dxfId="12" priority="2">
+    <cfRule type="expression" dxfId="5" priority="8">
       <formula>AND(MOD(ROW(),2)=0,$C2="Artiste")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="11" priority="3">
+    <cfRule type="expression" dxfId="4" priority="9">
       <formula>AND(MOD(ROW(),2)=1,$C2="Artiste")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="4">
+    <cfRule type="expression" dxfId="3" priority="10">
       <formula>AND(MOD(ROW(),2)=1,$C2="Junior.e")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="5">
+    <cfRule type="expression" dxfId="2" priority="11">
       <formula>AND(MOD(ROW(),2)=0,$C2="Junior.e")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="6">
+    <cfRule type="expression" dxfId="1" priority="12">
       <formula>AND(MOD(ROW(),2)=0,(OR($C2="Staff",$C2="Adjoint.e",$C2="COF")))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="7">
+    <cfRule type="expression" dxfId="0" priority="13">
       <formula>AND(MOD(ROW(),2)=1,(OR($C2="Staff",$C2="Adjoint.e",$C2="COF")))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L2:L3">
-    <cfRule type="expression" dxfId="6" priority="1">
-      <formula>$L$3=TRUE</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3577,10 +3791,10 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A29" t="str">
-        <v>Ledru</v>
+        <v>Jaquet</v>
       </c>
       <c r="B29" t="str">
-        <v>Lina-Rosa</v>
+        <v>Lisa</v>
       </c>
       <c r="C29" t="str">
         <v>Staff</v>
@@ -3591,7 +3805,7 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A30" t="str">
-        <v>Jaquet</v>
+        <v>Magnin</v>
       </c>
       <c r="B30" t="str">
         <v>Lisa</v>
@@ -3605,10 +3819,10 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A31" t="str">
-        <v>Magnin</v>
+        <v>Cardis</v>
       </c>
       <c r="B31" t="str">
-        <v>Lisa</v>
+        <v>Louis</v>
       </c>
       <c r="C31" t="str">
         <v>Staff</v>
@@ -3619,7 +3833,7 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A32" t="str">
-        <v>Cardis</v>
+        <v>Post</v>
       </c>
       <c r="B32" t="str">
         <v>Louis</v>
@@ -3633,13 +3847,13 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A33" t="str">
-        <v>Post</v>
+        <v>Blanchard</v>
       </c>
       <c r="B33" t="str">
-        <v>Louis</v>
+        <v>Louise</v>
       </c>
       <c r="C33" t="str">
-        <v>Staff</v>
+        <v>Adjoint.e</v>
       </c>
       <c r="D33" t="s">
         <v>14</v>
@@ -3647,13 +3861,13 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A34" t="str">
-        <v>Blanchard</v>
+        <v>Chastroux</v>
       </c>
       <c r="B34" t="str">
-        <v>Louise</v>
+        <v>Lucas</v>
       </c>
       <c r="C34" t="str">
-        <v>Adjoint.e</v>
+        <v>Staff</v>
       </c>
       <c r="D34" t="s">
         <v>8</v>
@@ -3661,10 +3875,10 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A35" t="str">
-        <v>Chastroux</v>
+        <v>Meyer</v>
       </c>
       <c r="B35" t="str">
-        <v>Lucas</v>
+        <v>Lucie</v>
       </c>
       <c r="C35" t="str">
         <v>Staff</v>
@@ -3675,10 +3889,10 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A36" t="str">
-        <v>Meyer</v>
+        <v>Ménétrey</v>
       </c>
       <c r="B36" t="str">
-        <v>Lucie</v>
+        <v>Maëlan</v>
       </c>
       <c r="C36" t="str">
         <v>Staff</v>
@@ -3689,13 +3903,13 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A37" t="str">
-        <v>Ménétrey</v>
+        <v>Chambaz</v>
       </c>
       <c r="B37" t="str">
-        <v>Maëlan</v>
+        <v>Maëlle</v>
       </c>
       <c r="C37" t="str">
-        <v>Staff</v>
+        <v>Adjoint.e</v>
       </c>
       <c r="D37" t="s">
         <v>14</v>
@@ -3703,13 +3917,13 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A38" t="str">
-        <v>Chambaz</v>
+        <v>Felix</v>
       </c>
       <c r="B38" t="str">
-        <v>Maëlle</v>
+        <v>Marius</v>
       </c>
       <c r="C38" t="str">
-        <v>Adjoint.e</v>
+        <v>Staff</v>
       </c>
       <c r="D38" t="s">
         <v>5</v>
@@ -3717,10 +3931,10 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A39" t="str">
-        <v>Felix</v>
+        <v>Ledru</v>
       </c>
       <c r="B39" t="str">
-        <v>Marius</v>
+        <v>Marot</v>
       </c>
       <c r="C39" t="str">
         <v>Staff</v>
@@ -3731,10 +3945,10 @@
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A40" t="str">
-        <v>Ledru</v>
+        <v>Cuinet</v>
       </c>
       <c r="B40" t="str">
-        <v>Marot</v>
+        <v>Mathis</v>
       </c>
       <c r="C40" t="str">
         <v>Staff</v>
@@ -3745,10 +3959,10 @@
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A41" t="str">
-        <v>Cuinet</v>
+        <v>Gavin</v>
       </c>
       <c r="B41" t="str">
-        <v>Mathis</v>
+        <v>Matteo</v>
       </c>
       <c r="C41" t="str">
         <v>Staff</v>
@@ -3759,10 +3973,10 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A42" t="str">
-        <v>Gavin</v>
+        <v>Debray</v>
       </c>
       <c r="B42" t="str">
-        <v>Matteo</v>
+        <v>Maxime</v>
       </c>
       <c r="C42" t="str">
         <v>Staff</v>
@@ -3773,10 +3987,10 @@
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A43" t="str">
-        <v>Debray</v>
+        <v>Corbelli</v>
       </c>
       <c r="B43" t="str">
-        <v>Maxime</v>
+        <v>Maya</v>
       </c>
       <c r="C43" t="str">
         <v>Staff</v>
@@ -3787,10 +4001,10 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A44" t="str">
-        <v>Corbelli</v>
+        <v>Pasche</v>
       </c>
       <c r="B44" t="str">
-        <v>Maya</v>
+        <v>Mickaël</v>
       </c>
       <c r="C44" t="str">
         <v>Staff</v>
@@ -3801,10 +4015,10 @@
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A45" t="str">
-        <v>Pasche</v>
+        <v>Ménard</v>
       </c>
       <c r="B45" t="str">
-        <v>Mickaël</v>
+        <v>Mireille</v>
       </c>
       <c r="C45" t="str">
         <v>Staff</v>
@@ -4046,11 +4260,11 @@
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A63" t="str">
-        <v>Ménard</v>
+      <c r="A63">
+        <v>0</v>
       </c>
       <c r="B63" t="str">
-        <v>Mireille</v>
+        <v>Andy</v>
       </c>
       <c r="C63" t="str">
         <v>Staff</v>
@@ -4078,22 +4292,22 @@
     <protectedRange sqref="D1:D1048576" name="Capacités"/>
   </protectedRanges>
   <conditionalFormatting sqref="A2:XFD67">
-    <cfRule type="expression" dxfId="5" priority="1">
+    <cfRule type="expression" dxfId="11" priority="1">
       <formula>AND(MOD(ROW(),2)=0,$C2="Artiste")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="2">
+    <cfRule type="expression" dxfId="10" priority="2">
       <formula>AND(MOD(ROW(),2)=1,$C2="Artiste")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="3">
+    <cfRule type="expression" dxfId="9" priority="3">
       <formula>AND(MOD(ROW(),2)=1,$C2="Junior.e")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="4">
+    <cfRule type="expression" dxfId="8" priority="4">
       <formula>AND(MOD(ROW(),2)=0,$C2="Junior.e")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="5">
+    <cfRule type="expression" dxfId="7" priority="5">
       <formula>AND(MOD(ROW(),2)=0,(OR($C2="Staff",$C2="Adjoint.e",$C2="COF")))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="6">
+    <cfRule type="expression" dxfId="6" priority="6">
       <formula>AND(MOD(ROW(),2)=1,(OR($C2="Staff",$C2="Adjoint.e",$C2="COF")))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>